<commit_message>
cleaned empty values in excel
</commit_message>
<xml_diff>
--- a/styleshop.xlsx
+++ b/styleshop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aryanbhandari/aryancoding/styleshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C516F6CD-418D-B945-832F-88DECE065C7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817AB88F-1E15-3C41-896A-CD8E5F5A6994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16140" xr2:uid="{296FE156-ABE8-A143-BE54-67E50949700F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="163">
   <si>
     <t>SKU</t>
   </si>
@@ -522,6 +522,12 @@
   </si>
   <si>
     <t>pine green</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pink </t>
+  </si>
+  <si>
+    <t>sweatshirt</t>
   </si>
 </sst>
 </file>
@@ -964,7 +970,7 @@
       </c>
       <c r="G2">
         <f ca="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>1699</v>
+        <v>1899</v>
       </c>
       <c r="H2">
         <f>ROW()+1000</f>
@@ -1006,7 +1012,7 @@
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G6" ca="1" si="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>899</v>
+        <v>1999</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H66" si="2">ROW()+1000</f>
@@ -1048,7 +1054,7 @@
       </c>
       <c r="G4">
         <f t="shared" ca="1" si="1"/>
-        <v>1999</v>
+        <v>1699</v>
       </c>
       <c r="H4">
         <f t="shared" si="2"/>
@@ -1090,7 +1096,7 @@
       </c>
       <c r="G5">
         <f t="shared" ca="1" si="1"/>
-        <v>999</v>
+        <v>1199</v>
       </c>
       <c r="H5">
         <f t="shared" si="2"/>
@@ -1174,7 +1180,7 @@
       </c>
       <c r="G7">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
-        <v>3899</v>
+        <v>3599</v>
       </c>
       <c r="H7">
         <f t="shared" si="2"/>
@@ -1216,7 +1222,7 @@
       </c>
       <c r="G8">
         <f t="shared" ref="G8:G13" ca="1" si="5">RANDBETWEEN(19,49)*100+99</f>
-        <v>2999</v>
+        <v>4599</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
@@ -1258,7 +1264,7 @@
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="5"/>
-        <v>3199</v>
+        <v>3099</v>
       </c>
       <c r="H9">
         <f t="shared" si="2"/>
@@ -1300,7 +1306,7 @@
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="5"/>
-        <v>2299</v>
+        <v>4999</v>
       </c>
       <c r="H10">
         <f t="shared" si="2"/>
@@ -1342,7 +1348,7 @@
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="5"/>
-        <v>4899</v>
+        <v>2399</v>
       </c>
       <c r="H11">
         <f t="shared" si="2"/>
@@ -1384,7 +1390,7 @@
       </c>
       <c r="G12">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
-        <v>3099</v>
+        <v>4599</v>
       </c>
       <c r="H12">
         <f t="shared" si="2"/>
@@ -1426,7 +1432,7 @@
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="5"/>
-        <v>3699</v>
+        <v>4799</v>
       </c>
       <c r="H13">
         <f t="shared" si="2"/>
@@ -1468,7 +1474,7 @@
       </c>
       <c r="G14">
         <f ca="1">RANDBETWEEN(7,49)*100+99</f>
-        <v>1899</v>
+        <v>4899</v>
       </c>
       <c r="H14">
         <f t="shared" si="2"/>
@@ -1509,7 +1515,7 @@
       </c>
       <c r="G15">
         <f t="shared" ref="G15:G78" ca="1" si="6">RANDBETWEEN(7,49)*100+99</f>
-        <v>4199</v>
+        <v>1299</v>
       </c>
       <c r="H15">
         <f t="shared" si="2"/>
@@ -1550,7 +1556,7 @@
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="6"/>
-        <v>2299</v>
+        <v>4299</v>
       </c>
       <c r="H16">
         <f t="shared" si="2"/>
@@ -1591,7 +1597,7 @@
       </c>
       <c r="G17">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>3999</v>
       </c>
       <c r="H17">
         <f t="shared" si="2"/>
@@ -1632,7 +1638,7 @@
       </c>
       <c r="G18">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>1099</v>
       </c>
       <c r="H18">
         <f t="shared" si="2"/>
@@ -1673,7 +1679,7 @@
       </c>
       <c r="G19">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>1099</v>
       </c>
       <c r="H19">
         <f t="shared" si="2"/>
@@ -1714,7 +1720,7 @@
       </c>
       <c r="G20">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>899</v>
       </c>
       <c r="H20">
         <f t="shared" si="2"/>
@@ -1756,7 +1762,7 @@
       </c>
       <c r="G21">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>3399</v>
       </c>
       <c r="H21">
         <f t="shared" si="2"/>
@@ -1798,7 +1804,7 @@
       </c>
       <c r="G22">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>3899</v>
       </c>
       <c r="H22">
         <f t="shared" si="2"/>
@@ -1840,7 +1846,7 @@
       </c>
       <c r="G23">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>3799</v>
       </c>
       <c r="H23">
         <f t="shared" si="2"/>
@@ -1882,7 +1888,7 @@
       </c>
       <c r="G24">
         <f t="shared" ca="1" si="6"/>
-        <v>2999</v>
+        <v>4099</v>
       </c>
       <c r="H24">
         <f t="shared" si="2"/>
@@ -1924,7 +1930,7 @@
       </c>
       <c r="G25">
         <f t="shared" ca="1" si="6"/>
-        <v>1899</v>
+        <v>4999</v>
       </c>
       <c r="H25">
         <f t="shared" si="2"/>
@@ -1966,7 +1972,7 @@
       </c>
       <c r="G26">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>1899</v>
       </c>
       <c r="H26">
         <f t="shared" si="2"/>
@@ -2008,7 +2014,7 @@
       </c>
       <c r="G27">
         <f t="shared" ca="1" si="6"/>
-        <v>3999</v>
+        <v>4999</v>
       </c>
       <c r="H27">
         <f t="shared" si="2"/>
@@ -2050,7 +2056,7 @@
       </c>
       <c r="G28">
         <f t="shared" ca="1" si="6"/>
-        <v>2599</v>
+        <v>4799</v>
       </c>
       <c r="H28">
         <f t="shared" si="2"/>
@@ -2092,7 +2098,7 @@
       </c>
       <c r="G29">
         <f t="shared" ca="1" si="6"/>
-        <v>1299</v>
+        <v>3899</v>
       </c>
       <c r="H29">
         <f t="shared" si="2"/>
@@ -2134,7 +2140,7 @@
       </c>
       <c r="G30">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>3199</v>
       </c>
       <c r="H30">
         <f t="shared" si="2"/>
@@ -2176,7 +2182,7 @@
       </c>
       <c r="G31">
         <f t="shared" ca="1" si="6"/>
-        <v>2199</v>
+        <v>2299</v>
       </c>
       <c r="H31">
         <f t="shared" si="2"/>
@@ -2218,7 +2224,7 @@
       </c>
       <c r="G32">
         <f t="shared" ca="1" si="6"/>
-        <v>899</v>
+        <v>4199</v>
       </c>
       <c r="H32">
         <f t="shared" si="2"/>
@@ -2260,7 +2266,7 @@
       </c>
       <c r="G33">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>2999</v>
       </c>
       <c r="H33">
         <f t="shared" si="2"/>
@@ -2302,7 +2308,7 @@
       </c>
       <c r="G34">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>1399</v>
       </c>
       <c r="H34">
         <f t="shared" si="2"/>
@@ -2344,7 +2350,7 @@
       </c>
       <c r="G35">
         <f t="shared" ca="1" si="6"/>
-        <v>4899</v>
+        <v>2699</v>
       </c>
       <c r="H35">
         <f t="shared" si="2"/>
@@ -2386,7 +2392,7 @@
       </c>
       <c r="G36">
         <f t="shared" ca="1" si="6"/>
-        <v>2699</v>
+        <v>899</v>
       </c>
       <c r="H36">
         <f t="shared" si="2"/>
@@ -2428,7 +2434,7 @@
       </c>
       <c r="G37">
         <f t="shared" ca="1" si="6"/>
-        <v>4899</v>
+        <v>4699</v>
       </c>
       <c r="H37">
         <f t="shared" si="2"/>
@@ -2470,7 +2476,7 @@
       </c>
       <c r="G38">
         <f t="shared" ca="1" si="6"/>
-        <v>1299</v>
+        <v>3999</v>
       </c>
       <c r="H38">
         <f t="shared" si="2"/>
@@ -2512,7 +2518,7 @@
       </c>
       <c r="G39">
         <f t="shared" ca="1" si="6"/>
-        <v>2599</v>
+        <v>4199</v>
       </c>
       <c r="H39">
         <f t="shared" si="2"/>
@@ -2540,6 +2546,9 @@
       <c r="B40" t="s">
         <v>48</v>
       </c>
+      <c r="C40" t="s">
+        <v>114</v>
+      </c>
       <c r="D40" t="s">
         <v>94</v>
       </c>
@@ -2551,7 +2560,7 @@
       </c>
       <c r="G40">
         <f t="shared" ca="1" si="6"/>
-        <v>1199</v>
+        <v>899</v>
       </c>
       <c r="H40">
         <f t="shared" si="2"/>
@@ -2578,6 +2587,9 @@
       <c r="B41" t="s">
         <v>49</v>
       </c>
+      <c r="C41" t="s">
+        <v>150</v>
+      </c>
       <c r="D41" t="s">
         <v>94</v>
       </c>
@@ -2589,7 +2601,7 @@
       </c>
       <c r="G41">
         <f t="shared" ca="1" si="6"/>
-        <v>2299</v>
+        <v>1099</v>
       </c>
       <c r="H41">
         <f t="shared" si="2"/>
@@ -2616,6 +2628,9 @@
       <c r="B42" t="s">
         <v>50</v>
       </c>
+      <c r="C42" t="s">
+        <v>154</v>
+      </c>
       <c r="D42" t="s">
         <v>94</v>
       </c>
@@ -2627,7 +2642,7 @@
       </c>
       <c r="G42">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>2399</v>
       </c>
       <c r="H42">
         <f t="shared" si="2"/>
@@ -2654,6 +2669,9 @@
       <c r="B43" t="s">
         <v>51</v>
       </c>
+      <c r="C43" t="s">
+        <v>148</v>
+      </c>
       <c r="D43" t="s">
         <v>94</v>
       </c>
@@ -2665,7 +2683,7 @@
       </c>
       <c r="G43">
         <f t="shared" ca="1" si="6"/>
-        <v>1499</v>
+        <v>1899</v>
       </c>
       <c r="H43">
         <f t="shared" si="2"/>
@@ -2692,6 +2710,9 @@
       <c r="B44" t="s">
         <v>52</v>
       </c>
+      <c r="C44" t="s">
+        <v>117</v>
+      </c>
       <c r="D44" t="s">
         <v>94</v>
       </c>
@@ -2703,7 +2724,7 @@
       </c>
       <c r="G44">
         <f t="shared" ca="1" si="6"/>
-        <v>1999</v>
+        <v>4799</v>
       </c>
       <c r="H44">
         <f t="shared" si="2"/>
@@ -2730,6 +2751,9 @@
       <c r="B45" t="s">
         <v>53</v>
       </c>
+      <c r="C45" t="s">
+        <v>114</v>
+      </c>
       <c r="D45" t="s">
         <v>94</v>
       </c>
@@ -2741,7 +2765,7 @@
       </c>
       <c r="G45">
         <f t="shared" ca="1" si="6"/>
-        <v>3799</v>
+        <v>2799</v>
       </c>
       <c r="H45">
         <f t="shared" si="2"/>
@@ -2769,6 +2793,9 @@
       <c r="B46" t="s">
         <v>54</v>
       </c>
+      <c r="C46" t="s">
+        <v>146</v>
+      </c>
       <c r="D46" t="s">
         <v>94</v>
       </c>
@@ -2780,7 +2807,7 @@
       </c>
       <c r="G46">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>2899</v>
       </c>
       <c r="H46">
         <f t="shared" si="2"/>
@@ -2808,6 +2835,9 @@
       <c r="B47" t="s">
         <v>55</v>
       </c>
+      <c r="C47" t="s">
+        <v>133</v>
+      </c>
       <c r="D47" t="s">
         <v>94</v>
       </c>
@@ -2819,7 +2849,7 @@
       </c>
       <c r="G47">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>3699</v>
       </c>
       <c r="H47">
         <f t="shared" si="2"/>
@@ -2847,6 +2877,9 @@
       <c r="B48" t="s">
         <v>56</v>
       </c>
+      <c r="C48" t="s">
+        <v>114</v>
+      </c>
       <c r="D48" t="s">
         <v>94</v>
       </c>
@@ -2858,15 +2891,14 @@
       </c>
       <c r="G48">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>899</v>
       </c>
       <c r="H48">
         <f t="shared" si="2"/>
         <v>1048</v>
       </c>
-      <c r="I48" t="str">
-        <f t="shared" si="3"/>
-        <v>sweat</v>
+      <c r="I48" t="s">
+        <v>162</v>
       </c>
       <c r="J48">
         <v>5</v>
@@ -2886,6 +2918,9 @@
       <c r="B49" t="s">
         <v>57</v>
       </c>
+      <c r="C49" t="s">
+        <v>133</v>
+      </c>
       <c r="D49" t="s">
         <v>94</v>
       </c>
@@ -2897,15 +2932,14 @@
       </c>
       <c r="G49">
         <f t="shared" ca="1" si="6"/>
-        <v>2799</v>
+        <v>2399</v>
       </c>
       <c r="H49">
         <f t="shared" si="2"/>
         <v>1049</v>
       </c>
-      <c r="I49" t="str">
-        <f t="shared" si="3"/>
-        <v>sweat</v>
+      <c r="I49" t="s">
+        <v>162</v>
       </c>
       <c r="J49">
         <v>5</v>
@@ -2925,6 +2959,9 @@
       <c r="B50" t="s">
         <v>58</v>
       </c>
+      <c r="C50" t="s">
+        <v>136</v>
+      </c>
       <c r="D50" t="s">
         <v>94</v>
       </c>
@@ -2936,7 +2973,7 @@
       </c>
       <c r="G50">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>2399</v>
       </c>
       <c r="H50">
         <f t="shared" si="2"/>
@@ -2964,6 +3001,9 @@
       <c r="B51" t="s">
         <v>59</v>
       </c>
+      <c r="C51" t="s">
+        <v>117</v>
+      </c>
       <c r="D51" t="s">
         <v>94</v>
       </c>
@@ -2975,7 +3015,7 @@
       </c>
       <c r="G51">
         <f t="shared" ca="1" si="6"/>
-        <v>1399</v>
+        <v>799</v>
       </c>
       <c r="H51">
         <f t="shared" si="2"/>
@@ -3003,6 +3043,9 @@
       <c r="B52" t="s">
         <v>60</v>
       </c>
+      <c r="C52" t="s">
+        <v>146</v>
+      </c>
       <c r="D52" t="s">
         <v>94</v>
       </c>
@@ -3014,7 +3057,7 @@
       </c>
       <c r="G52">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>999</v>
       </c>
       <c r="H52">
         <f t="shared" si="2"/>
@@ -3042,6 +3085,9 @@
       <c r="B53" t="s">
         <v>61</v>
       </c>
+      <c r="C53" t="s">
+        <v>161</v>
+      </c>
       <c r="D53" t="s">
         <v>94</v>
       </c>
@@ -3053,7 +3099,7 @@
       </c>
       <c r="G53">
         <f t="shared" ca="1" si="6"/>
-        <v>2299</v>
+        <v>3099</v>
       </c>
       <c r="H53">
         <f t="shared" si="2"/>
@@ -3090,9 +3136,12 @@
       <c r="E54" t="s">
         <v>97</v>
       </c>
+      <c r="F54" t="s">
+        <v>119</v>
+      </c>
       <c r="G54">
         <f t="shared" ca="1" si="6"/>
-        <v>3199</v>
+        <v>4799</v>
       </c>
       <c r="H54">
         <f t="shared" si="2"/>
@@ -3133,7 +3182,7 @@
       </c>
       <c r="G55">
         <f t="shared" ca="1" si="6"/>
-        <v>2399</v>
+        <v>4199</v>
       </c>
       <c r="H55">
         <f t="shared" si="2"/>
@@ -3174,7 +3223,7 @@
       </c>
       <c r="G56">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>4999</v>
       </c>
       <c r="H56">
         <f t="shared" si="2"/>
@@ -3215,7 +3264,7 @@
       </c>
       <c r="G57">
         <f t="shared" ca="1" si="6"/>
-        <v>1499</v>
+        <v>3899</v>
       </c>
       <c r="H57">
         <f t="shared" si="2"/>
@@ -3251,9 +3300,12 @@
       <c r="E58" t="s">
         <v>98</v>
       </c>
+      <c r="F58" t="s">
+        <v>119</v>
+      </c>
       <c r="G58">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>3199</v>
       </c>
       <c r="H58">
         <f t="shared" si="2"/>
@@ -3289,9 +3341,12 @@
       <c r="E59" t="s">
         <v>107</v>
       </c>
+      <c r="F59" t="s">
+        <v>119</v>
+      </c>
       <c r="G59">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>3699</v>
       </c>
       <c r="H59">
         <f t="shared" si="2"/>
@@ -3329,7 +3384,7 @@
       </c>
       <c r="G60">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>2399</v>
       </c>
       <c r="H60">
         <f t="shared" si="2"/>
@@ -3365,9 +3420,12 @@
       <c r="E61" t="s">
         <v>110</v>
       </c>
+      <c r="F61" t="s">
+        <v>119</v>
+      </c>
       <c r="G61">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>1799</v>
       </c>
       <c r="H61">
         <f t="shared" si="2"/>
@@ -3403,9 +3461,12 @@
       <c r="E62" t="s">
         <v>99</v>
       </c>
+      <c r="F62" t="s">
+        <v>119</v>
+      </c>
       <c r="G62">
         <f t="shared" ca="1" si="6"/>
-        <v>3999</v>
+        <v>4599</v>
       </c>
       <c r="H62">
         <f t="shared" si="2"/>
@@ -3441,9 +3502,12 @@
       <c r="E63" t="s">
         <v>112</v>
       </c>
+      <c r="F63" t="s">
+        <v>119</v>
+      </c>
       <c r="G63">
         <f t="shared" ca="1" si="6"/>
-        <v>2099</v>
+        <v>3899</v>
       </c>
       <c r="H63">
         <f t="shared" si="2"/>
@@ -3481,7 +3545,7 @@
       </c>
       <c r="G64">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>4799</v>
       </c>
       <c r="H64">
         <f t="shared" si="2"/>
@@ -3516,7 +3580,7 @@
       </c>
       <c r="G65">
         <f t="shared" ca="1" si="6"/>
-        <v>4999</v>
+        <v>3199</v>
       </c>
       <c r="H65">
         <f t="shared" si="2"/>
@@ -3549,13 +3613,19 @@
       <c r="E66" t="s">
         <v>105</v>
       </c>
+      <c r="F66" t="s">
+        <v>119</v>
+      </c>
       <c r="G66">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>1999</v>
       </c>
       <c r="H66">
         <f t="shared" si="2"/>
         <v>1066</v>
+      </c>
+      <c r="I66" t="s">
+        <v>94</v>
       </c>
       <c r="J66">
         <v>3</v>
@@ -3586,7 +3656,7 @@
       </c>
       <c r="G67">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>3399</v>
       </c>
       <c r="H67">
         <f t="shared" ref="H67:H79" si="7">ROW()+1000</f>
@@ -3622,14 +3692,20 @@
       <c r="E68" t="s">
         <v>106</v>
       </c>
+      <c r="F68" t="s">
+        <v>119</v>
+      </c>
       <c r="G68">
         <f t="shared" ca="1" si="6"/>
-        <v>1999</v>
+        <v>899</v>
       </c>
       <c r="H68">
         <f t="shared" si="7"/>
         <v>1068</v>
       </c>
+      <c r="I68" t="s">
+        <v>94</v>
+      </c>
       <c r="J68">
         <v>3</v>
       </c>
@@ -3659,7 +3735,7 @@
       </c>
       <c r="G69">
         <f t="shared" ca="1" si="6"/>
-        <v>4899</v>
+        <v>3399</v>
       </c>
       <c r="H69">
         <f t="shared" si="7"/>
@@ -3694,7 +3770,7 @@
       </c>
       <c r="G70">
         <f t="shared" ca="1" si="6"/>
-        <v>3399</v>
+        <v>2599</v>
       </c>
       <c r="H70">
         <f t="shared" si="7"/>
@@ -3727,13 +3803,19 @@
       <c r="E71" t="s">
         <v>110</v>
       </c>
+      <c r="F71" t="s">
+        <v>119</v>
+      </c>
       <c r="G71">
         <f t="shared" ca="1" si="6"/>
-        <v>1499</v>
+        <v>1699</v>
       </c>
       <c r="H71">
         <f t="shared" si="7"/>
         <v>1071</v>
+      </c>
+      <c r="I71" t="s">
+        <v>126</v>
       </c>
       <c r="J71">
         <v>3</v>
@@ -3762,9 +3844,12 @@
       <c r="E72" t="s">
         <v>104</v>
       </c>
+      <c r="F72" t="s">
+        <v>119</v>
+      </c>
       <c r="G72">
         <f t="shared" ca="1" si="6"/>
-        <v>4299</v>
+        <v>2699</v>
       </c>
       <c r="H72">
         <f t="shared" si="7"/>
@@ -3802,7 +3887,7 @@
       </c>
       <c r="G73">
         <f t="shared" ca="1" si="6"/>
-        <v>4899</v>
+        <v>1499</v>
       </c>
       <c r="H73">
         <f t="shared" si="7"/>
@@ -3838,9 +3923,12 @@
       <c r="E74" t="s">
         <v>105</v>
       </c>
+      <c r="F74" t="s">
+        <v>119</v>
+      </c>
       <c r="G74">
         <f t="shared" ca="1" si="6"/>
-        <v>1999</v>
+        <v>2199</v>
       </c>
       <c r="H74">
         <f t="shared" si="7"/>
@@ -3876,9 +3964,12 @@
       <c r="E75" t="s">
         <v>99</v>
       </c>
+      <c r="F75" t="s">
+        <v>119</v>
+      </c>
       <c r="G75">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>2199</v>
       </c>
       <c r="H75">
         <f t="shared" si="7"/>
@@ -3914,13 +4005,19 @@
       <c r="E76" t="s">
         <v>106</v>
       </c>
+      <c r="F76" t="s">
+        <v>119</v>
+      </c>
       <c r="G76">
         <f t="shared" ca="1" si="6"/>
-        <v>2699</v>
+        <v>4399</v>
       </c>
       <c r="H76">
         <f t="shared" si="7"/>
         <v>1076</v>
+      </c>
+      <c r="I76" t="s">
+        <v>94</v>
       </c>
       <c r="J76">
         <v>6</v>
@@ -3951,7 +4048,7 @@
       </c>
       <c r="G77">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>1599</v>
       </c>
       <c r="H77">
         <f t="shared" si="7"/>
@@ -3987,9 +4084,12 @@
       <c r="E78" t="s">
         <v>102</v>
       </c>
+      <c r="F78" t="s">
+        <v>119</v>
+      </c>
       <c r="G78">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>4299</v>
       </c>
       <c r="H78">
         <f t="shared" si="7"/>
@@ -4025,9 +4125,12 @@
       <c r="E79" t="s">
         <v>105</v>
       </c>
+      <c r="F79" t="s">
+        <v>119</v>
+      </c>
       <c r="G79">
         <f t="shared" ref="G79:G83" ca="1" si="9">RANDBETWEEN(7,49)*100+99</f>
-        <v>3999</v>
+        <v>3499</v>
       </c>
       <c r="H79">
         <f t="shared" si="7"/>
@@ -4065,7 +4168,7 @@
       </c>
       <c r="G80">
         <f t="shared" ca="1" si="9"/>
-        <v>4399</v>
+        <v>4199</v>
       </c>
       <c r="H80">
         <f>ROW()+1000</f>
@@ -4101,9 +4204,12 @@
       <c r="E81" t="s">
         <v>113</v>
       </c>
+      <c r="F81" t="s">
+        <v>119</v>
+      </c>
       <c r="G81">
         <f t="shared" ca="1" si="9"/>
-        <v>1699</v>
+        <v>3199</v>
       </c>
       <c r="H81">
         <f t="shared" ref="H81:H83" si="10">ROW()+1000</f>
@@ -4139,9 +4245,12 @@
       <c r="E82" t="s">
         <v>105</v>
       </c>
+      <c r="F82" t="s">
+        <v>119</v>
+      </c>
       <c r="G82">
         <f t="shared" ca="1" si="9"/>
-        <v>2199</v>
+        <v>3699</v>
       </c>
       <c r="H82">
         <f t="shared" si="10"/>
@@ -4177,9 +4286,12 @@
       <c r="E83" t="s">
         <v>105</v>
       </c>
+      <c r="F83" t="s">
+        <v>119</v>
+      </c>
       <c r="G83">
         <f t="shared" ca="1" si="9"/>
-        <v>4499</v>
+        <v>3599</v>
       </c>
       <c r="H83">
         <f t="shared" si="10"/>

</xml_diff>

<commit_message>
added values in excel
</commit_message>
<xml_diff>
--- a/styleshop.xlsx
+++ b/styleshop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aryanbhandari/aryancoding/styleshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE68C77-E3C5-5348-9AA5-0BD94D05B5CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884DC111-4A38-3E42-8F7A-51285E6974E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{296FE156-ABE8-A143-BE54-67E50949700F}"/>
   </bookViews>
@@ -39,14 +39,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="178">
   <si>
     <t>SKU</t>
   </si>
   <si>
-    <t>gender</t>
-  </si>
-  <si>
     <t>category</t>
   </si>
   <si>
@@ -104,9 +101,6 @@
     <t>formalshirt_lightb.jpg</t>
   </si>
   <si>
-    <t>formalshirt_pink.jpg</t>
-  </si>
-  <si>
     <t>graphic_black.jpg</t>
   </si>
   <si>
@@ -528,6 +522,57 @@
   </si>
   <si>
     <t>sweatshirt</t>
+  </si>
+  <si>
+    <t>formalshirt_white.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gender = male </t>
+  </si>
+  <si>
+    <t>black formal pants.avif</t>
+  </si>
+  <si>
+    <t>blue croptop.avif</t>
+  </si>
+  <si>
+    <t>halter neck sequined.avif</t>
+  </si>
+  <si>
+    <t>khaki green formal trouser.avif</t>
+  </si>
+  <si>
+    <t>light blue full sleeve shirt.avif</t>
+  </si>
+  <si>
+    <t>pink flounced blouse.avif</t>
+  </si>
+  <si>
+    <t>pink tank top.avif</t>
+  </si>
+  <si>
+    <t>red fine knit.jpeg</t>
+  </si>
+  <si>
+    <t>red halter.avif</t>
+  </si>
+  <si>
+    <t>red peplum.avif</t>
+  </si>
+  <si>
+    <t>white formal pants.avif</t>
+  </si>
+  <si>
+    <t>yellow top.avif</t>
+  </si>
+  <si>
+    <t>pants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blue </t>
+  </si>
+  <si>
+    <t xml:space="preserve">formal </t>
   </si>
 </sst>
 </file>
@@ -899,7 +944,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC477210-8802-4647-A9A0-82022E3B188B}">
-  <dimension ref="A1:L83"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="130.6640625" customWidth="1"/>
@@ -911,40 +957,40 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" t="s">
         <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>158</v>
-      </c>
-      <c r="F1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" t="s">
-        <v>3</v>
       </c>
       <c r="H1" t="s">
         <v>0</v>
       </c>
       <c r="I1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
-        <v>7</v>
-      </c>
       <c r="L1" t="s">
-        <v>1</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -953,23 +999,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/casual_black.jpg</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G2">
         <f ca="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>1599</v>
+        <v>1999</v>
       </c>
       <c r="H2">
         <f>ROW()+1000</f>
@@ -986,7 +1032,7 @@
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -995,23 +1041,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/casual_earthy.jpg</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G6" ca="1" si="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>1399</v>
+        <v>1899</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H66" si="2">ROW()+1000</f>
@@ -1028,7 +1074,7 @@
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
@@ -1037,23 +1083,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/casual_pastel.jpg</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G4">
         <f t="shared" ca="1" si="1"/>
-        <v>1199</v>
+        <v>1899</v>
       </c>
       <c r="H4">
         <f t="shared" si="2"/>
@@ -1070,7 +1116,7 @@
         <v>1</v>
       </c>
       <c r="L4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -1079,19 +1125,19 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/casual_pastel1.jpg</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F5" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G5">
         <f t="shared" ca="1" si="1"/>
@@ -1112,7 +1158,7 @@
         <v>1</v>
       </c>
       <c r="L5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -1121,23 +1167,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/casual_white.jpg</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G6">
         <f t="shared" ca="1" si="1"/>
-        <v>1299</v>
+        <v>1399</v>
       </c>
       <c r="H6">
         <f t="shared" si="2"/>
@@ -1154,28 +1200,28 @@
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="str">
         <f t="shared" si="0"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formals_beige.jpg</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G7">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
@@ -1196,32 +1242,32 @@
         <v>1</v>
       </c>
       <c r="L7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="str">
         <f t="shared" ref="A8:A71" si="4">"https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/" &amp; B8</f>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formals_black.jpg</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E8" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G8">
         <f t="shared" ref="G8:G13" ca="1" si="5">RANDBETWEEN(19,49)*100+99</f>
-        <v>2599</v>
+        <v>3099</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
@@ -1238,32 +1284,32 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formals_grey.jpg</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="5"/>
-        <v>4799</v>
+        <v>4699</v>
       </c>
       <c r="H9">
         <f t="shared" si="2"/>
@@ -1280,32 +1326,32 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formals_navy.jpg</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="5"/>
-        <v>2099</v>
+        <v>2899</v>
       </c>
       <c r="H10">
         <f t="shared" si="2"/>
@@ -1322,28 +1368,28 @@
         <v>1</v>
       </c>
       <c r="L10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formals_white.jpg</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E11" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="5"/>
@@ -1364,7 +1410,7 @@
         <v>1</v>
       </c>
       <c r="L11" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
@@ -1373,23 +1419,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formalshirt_lightb.jpg</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G12">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
-        <v>2899</v>
+        <v>2499</v>
       </c>
       <c r="H12">
         <f t="shared" si="2"/>
@@ -1406,32 +1452,32 @@
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
         <f t="shared" si="4"/>
-        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formalshirt_pink.jpg</v>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formalshirt_white.jpg</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>161</v>
       </c>
       <c r="C13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="5"/>
-        <v>4699</v>
+        <v>3499</v>
       </c>
       <c r="H13">
         <f t="shared" si="2"/>
@@ -1448,7 +1494,7 @@
         <v>1</v>
       </c>
       <c r="L13" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
@@ -1457,30 +1503,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/graphic_black.jpg</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D14" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" t="s">
         <v>94</v>
       </c>
-      <c r="E14" t="s">
-        <v>96</v>
-      </c>
       <c r="F14" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G14">
         <f ca="1">RANDBETWEEN(7,49)*100+99</f>
-        <v>4499</v>
+        <v>2099</v>
       </c>
       <c r="H14">
         <f t="shared" si="2"/>
         <v>1014</v>
       </c>
       <c r="I14" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J14">
         <v>2</v>
@@ -1489,7 +1535,7 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
@@ -1498,30 +1544,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/graphic_bright.jpg</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D15" t="s">
+        <v>92</v>
+      </c>
+      <c r="E15" t="s">
         <v>94</v>
       </c>
-      <c r="E15" t="s">
-        <v>96</v>
-      </c>
       <c r="F15" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G15">
         <f t="shared" ref="G15:G78" ca="1" si="6">RANDBETWEEN(7,49)*100+99</f>
-        <v>3899</v>
+        <v>3999</v>
       </c>
       <c r="H15">
         <f t="shared" si="2"/>
         <v>1015</v>
       </c>
       <c r="I15" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J15">
         <v>2</v>
@@ -1530,7 +1576,7 @@
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
@@ -1539,30 +1585,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/graphic_earthy.jpg</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E16" t="s">
         <v>94</v>
       </c>
-      <c r="E16" t="s">
-        <v>96</v>
-      </c>
       <c r="F16" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="6"/>
-        <v>3399</v>
+        <v>799</v>
       </c>
       <c r="H16">
         <f t="shared" si="2"/>
         <v>1016</v>
       </c>
       <c r="I16" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1571,7 +1617,7 @@
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
@@ -1580,30 +1626,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/graphic_navy.jpg</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D17" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" t="s">
         <v>94</v>
       </c>
-      <c r="E17" t="s">
-        <v>96</v>
-      </c>
       <c r="F17" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G17">
         <f t="shared" ca="1" si="6"/>
-        <v>1299</v>
+        <v>3199</v>
       </c>
       <c r="H17">
         <f t="shared" si="2"/>
         <v>1017</v>
       </c>
       <c r="I17" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J17">
         <v>2</v>
@@ -1612,7 +1658,7 @@
         <v>1</v>
       </c>
       <c r="L17" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
@@ -1621,30 +1667,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/graphic_pastel.jpg</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D18" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" t="s">
         <v>94</v>
       </c>
-      <c r="E18" t="s">
-        <v>96</v>
-      </c>
       <c r="F18" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G18">
         <f t="shared" ca="1" si="6"/>
-        <v>1999</v>
+        <v>1599</v>
       </c>
       <c r="H18">
         <f t="shared" si="2"/>
         <v>1018</v>
       </c>
       <c r="I18" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J18">
         <v>2</v>
@@ -1653,7 +1699,7 @@
         <v>1</v>
       </c>
       <c r="L18" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
@@ -1662,19 +1708,19 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/graphic_white.jpg</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" t="s">
         <v>94</v>
       </c>
-      <c r="E19" t="s">
-        <v>96</v>
-      </c>
       <c r="F19" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G19">
         <f t="shared" ca="1" si="6"/>
@@ -1685,7 +1731,7 @@
         <v>1019</v>
       </c>
       <c r="I19" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J19">
         <v>4</v>
@@ -1694,7 +1740,7 @@
         <v>1</v>
       </c>
       <c r="L19" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
@@ -1703,23 +1749,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/hoodie_black.jpg</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D20" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" t="s">
         <v>94</v>
       </c>
-      <c r="E20" t="s">
-        <v>96</v>
-      </c>
       <c r="F20" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G20">
         <f t="shared" ca="1" si="6"/>
-        <v>4099</v>
+        <v>1599</v>
       </c>
       <c r="H20">
         <f t="shared" si="2"/>
@@ -1736,7 +1782,7 @@
         <v>1</v>
       </c>
       <c r="L20" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
@@ -1745,23 +1791,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/hoodie_blue bright.jpg</v>
       </c>
       <c r="B21" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D21" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" t="s">
         <v>94</v>
       </c>
-      <c r="E21" t="s">
-        <v>96</v>
-      </c>
       <c r="F21" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G21">
         <f t="shared" ca="1" si="6"/>
-        <v>4899</v>
+        <v>4699</v>
       </c>
       <c r="H21">
         <f t="shared" si="2"/>
@@ -1778,7 +1824,7 @@
         <v>1</v>
       </c>
       <c r="L21" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.2">
@@ -1787,23 +1833,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/hoodie_earthyg.jpg</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D22" t="s">
+        <v>92</v>
+      </c>
+      <c r="E22" t="s">
         <v>94</v>
       </c>
-      <c r="E22" t="s">
-        <v>96</v>
-      </c>
       <c r="F22" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G22">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>1699</v>
       </c>
       <c r="H22">
         <f t="shared" si="2"/>
@@ -1820,32 +1866,32 @@
         <v>1</v>
       </c>
       <c r="L22" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/jacket_black.jpg</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D23" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G23">
         <f t="shared" ca="1" si="6"/>
-        <v>999</v>
+        <v>3799</v>
       </c>
       <c r="H23">
         <f t="shared" si="2"/>
@@ -1862,32 +1908,32 @@
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/jacket_lightb.jpg</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C24" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D24" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F24" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G24">
         <f t="shared" ca="1" si="6"/>
-        <v>1799</v>
+        <v>2499</v>
       </c>
       <c r="H24">
         <f t="shared" si="2"/>
@@ -1904,32 +1950,32 @@
         <v>1</v>
       </c>
       <c r="L24" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/jacket_ochre.jpg</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D25" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F25" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G25">
         <f t="shared" ca="1" si="6"/>
-        <v>3999</v>
+        <v>4999</v>
       </c>
       <c r="H25">
         <f t="shared" si="2"/>
@@ -1946,32 +1992,32 @@
         <v>1</v>
       </c>
       <c r="L25" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/jeans_black.jpg</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E26" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F26" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G26">
         <f t="shared" ca="1" si="6"/>
-        <v>1199</v>
+        <v>3099</v>
       </c>
       <c r="H26">
         <f t="shared" si="2"/>
@@ -1988,32 +2034,32 @@
         <v>1</v>
       </c>
       <c r="L26" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/jeans_darkb.jpg</v>
       </c>
       <c r="B27" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D27" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F27" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G27">
         <f t="shared" ca="1" si="6"/>
-        <v>3599</v>
+        <v>4799</v>
       </c>
       <c r="H27">
         <f t="shared" si="2"/>
@@ -2030,32 +2076,32 @@
         <v>1</v>
       </c>
       <c r="L27" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/jeans_grey.jpg</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C28" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D28" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E28" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F28" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G28">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>1199</v>
       </c>
       <c r="H28">
         <f t="shared" si="2"/>
@@ -2072,32 +2118,32 @@
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/jeans_lighb.jpg</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D29" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E29" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F29" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G29">
         <f t="shared" ca="1" si="6"/>
-        <v>4699</v>
+        <v>3099</v>
       </c>
       <c r="H29">
         <f t="shared" si="2"/>
@@ -2114,7 +2160,7 @@
         <v>1</v>
       </c>
       <c r="L29" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
@@ -2123,23 +2169,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/overshirt_black.jpg</v>
       </c>
       <c r="B30" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E30" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F30" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G30">
         <f t="shared" ca="1" si="6"/>
-        <v>1999</v>
+        <v>2799</v>
       </c>
       <c r="H30">
         <f t="shared" si="2"/>
@@ -2156,7 +2202,7 @@
         <v>1</v>
       </c>
       <c r="L30" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.2">
@@ -2165,23 +2211,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/overshirt_olive.jpg</v>
       </c>
       <c r="B31" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D31" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E31" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F31" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G31">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>2799</v>
       </c>
       <c r="H31">
         <f t="shared" si="2"/>
@@ -2198,7 +2244,7 @@
         <v>1</v>
       </c>
       <c r="L31" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
@@ -2207,23 +2253,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/overshirt_red.jpg</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D32" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E32" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F32" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G32">
         <f t="shared" ca="1" si="6"/>
-        <v>1799</v>
+        <v>3399</v>
       </c>
       <c r="H32">
         <f t="shared" si="2"/>
@@ -2240,7 +2286,7 @@
         <v>1</v>
       </c>
       <c r="L32" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
@@ -2249,23 +2295,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/polo_black.jpg</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D33" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E33" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F33" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G33">
         <f t="shared" ca="1" si="6"/>
-        <v>2099</v>
+        <v>2799</v>
       </c>
       <c r="H33">
         <f t="shared" si="2"/>
@@ -2282,7 +2328,7 @@
         <v>1</v>
       </c>
       <c r="L33" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.2">
@@ -2291,23 +2337,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/polo_earthy.jpg</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D34" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E34" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F34" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G34">
         <f t="shared" ca="1" si="6"/>
-        <v>2699</v>
+        <v>3699</v>
       </c>
       <c r="H34">
         <f t="shared" si="2"/>
@@ -2324,7 +2370,7 @@
         <v>1</v>
       </c>
       <c r="L34" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
@@ -2333,23 +2379,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/polo_purple.jpg</v>
       </c>
       <c r="B35" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D35" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E35" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F35" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G35">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>3899</v>
       </c>
       <c r="H35">
         <f t="shared" si="2"/>
@@ -2366,7 +2412,7 @@
         <v>1</v>
       </c>
       <c r="L35" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
@@ -2375,23 +2421,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/polo_white.jpg</v>
       </c>
       <c r="B36" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D36" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E36" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F36" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G36">
         <f t="shared" ca="1" si="6"/>
-        <v>1599</v>
+        <v>2399</v>
       </c>
       <c r="H36">
         <f t="shared" si="2"/>
@@ -2408,32 +2454,32 @@
         <v>1</v>
       </c>
       <c r="L36" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/shorts_black.jpg</v>
       </c>
       <c r="B37" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C37" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D37" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E37" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F37" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G37">
         <f t="shared" ca="1" si="6"/>
-        <v>3299</v>
+        <v>999</v>
       </c>
       <c r="H37">
         <f t="shared" si="2"/>
@@ -2450,32 +2496,32 @@
         <v>1</v>
       </c>
       <c r="L37" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/shorts_lightb.jpg</v>
       </c>
       <c r="B38" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C38" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D38" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E38" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F38" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G38">
         <f t="shared" ca="1" si="6"/>
-        <v>999</v>
+        <v>799</v>
       </c>
       <c r="H38">
         <f t="shared" si="2"/>
@@ -2492,32 +2538,32 @@
         <v>1</v>
       </c>
       <c r="L38" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="str">
         <f t="shared" si="4"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/shorts_white.jpg</v>
       </c>
       <c r="B39" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C39" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D39" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E39" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F39" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G39">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>2399</v>
       </c>
       <c r="H39">
         <f t="shared" si="2"/>
@@ -2534,7 +2580,7 @@
         <v>1</v>
       </c>
       <c r="L39" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.2">
@@ -2543,30 +2589,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/solids_black.jpg</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C40" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D40" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E40" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F40" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G40">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>4199</v>
       </c>
       <c r="H40">
         <f t="shared" si="2"/>
         <v>1040</v>
       </c>
       <c r="I40" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J40">
         <v>7</v>
@@ -2575,7 +2621,7 @@
         <v>1</v>
       </c>
       <c r="L40" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.2">
@@ -2584,30 +2630,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/solids_bright.jpg</v>
       </c>
       <c r="B41" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C41" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D41" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E41" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F41" t="s">
+        <v>117</v>
+      </c>
+      <c r="G41">
+        <f t="shared" ca="1" si="6"/>
+        <v>999</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="2"/>
+        <v>1041</v>
+      </c>
+      <c r="I41" t="s">
         <v>119</v>
-      </c>
-      <c r="G41">
-        <f t="shared" ca="1" si="6"/>
-        <v>1499</v>
-      </c>
-      <c r="H41">
-        <f t="shared" si="2"/>
-        <v>1041</v>
-      </c>
-      <c r="I41" t="s">
-        <v>121</v>
       </c>
       <c r="J41">
         <v>7</v>
@@ -2616,7 +2662,7 @@
         <v>1</v>
       </c>
       <c r="L41" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.2">
@@ -2625,30 +2671,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/solids_earthy.jpg</v>
       </c>
       <c r="B42" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C42" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D42" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E42" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F42" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G42">
         <f t="shared" ca="1" si="6"/>
-        <v>899</v>
+        <v>3599</v>
       </c>
       <c r="H42">
         <f t="shared" si="2"/>
         <v>1042</v>
       </c>
       <c r="I42" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J42">
         <v>7</v>
@@ -2657,7 +2703,7 @@
         <v>1</v>
       </c>
       <c r="L42" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.2">
@@ -2666,30 +2712,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/solids_pastel.jpg</v>
       </c>
       <c r="B43" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D43" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E43" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F43" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G43">
         <f t="shared" ca="1" si="6"/>
-        <v>4099</v>
+        <v>1899</v>
       </c>
       <c r="H43">
         <f t="shared" si="2"/>
         <v>1043</v>
       </c>
       <c r="I43" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J43">
         <v>7</v>
@@ -2698,7 +2744,7 @@
         <v>1</v>
       </c>
       <c r="L43" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
@@ -2707,30 +2753,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/solids_white.jpg</v>
       </c>
       <c r="B44" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C44" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D44" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E44" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F44" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G44">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>2499</v>
       </c>
       <c r="H44">
         <f t="shared" si="2"/>
         <v>1044</v>
       </c>
       <c r="I44" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J44">
         <v>5</v>
@@ -2739,7 +2785,7 @@
         <v>1</v>
       </c>
       <c r="L44" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
@@ -2748,23 +2794,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/suits_black.jpg</v>
       </c>
       <c r="B45" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C45" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D45" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E45" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F45" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G45">
         <f t="shared" ca="1" si="6"/>
-        <v>4499</v>
+        <v>2099</v>
       </c>
       <c r="H45">
         <f t="shared" si="2"/>
@@ -2781,7 +2827,7 @@
         <v>1</v>
       </c>
       <c r="L45" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
@@ -2790,23 +2836,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/suits_bright.jpg</v>
       </c>
       <c r="B46" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C46" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D46" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E46" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F46" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G46">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>4399</v>
       </c>
       <c r="H46">
         <f t="shared" si="2"/>
@@ -2823,7 +2869,7 @@
         <v>1</v>
       </c>
       <c r="L46" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
@@ -2832,23 +2878,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/suits_earthy.jpg</v>
       </c>
       <c r="B47" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C47" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D47" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E47" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F47" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G47">
         <f t="shared" ca="1" si="6"/>
-        <v>2099</v>
+        <v>4599</v>
       </c>
       <c r="H47">
         <f t="shared" si="2"/>
@@ -2865,7 +2911,7 @@
         <v>1</v>
       </c>
       <c r="L47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
@@ -2874,30 +2920,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/sweat_black.jpg</v>
       </c>
       <c r="B48" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C48" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D48" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E48" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F48" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G48">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>799</v>
       </c>
       <c r="H48">
         <f t="shared" si="2"/>
         <v>1048</v>
       </c>
       <c r="I48" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J48">
         <v>5</v>
@@ -2906,7 +2952,7 @@
         <v>1</v>
       </c>
       <c r="L48" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
@@ -2915,30 +2961,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/sweat_grey.jpg</v>
       </c>
       <c r="B49" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C49" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D49" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E49" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F49" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G49">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>3799</v>
       </c>
       <c r="H49">
         <f t="shared" si="2"/>
         <v>1049</v>
       </c>
       <c r="I49" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="J49">
         <v>5</v>
@@ -2947,7 +2993,7 @@
         <v>1</v>
       </c>
       <c r="L49" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
@@ -2956,23 +3002,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/sweater_pastel.jpg</v>
       </c>
       <c r="B50" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C50" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D50" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E50" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F50" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G50">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>1399</v>
       </c>
       <c r="H50">
         <f t="shared" si="2"/>
@@ -2989,7 +3035,7 @@
         <v>1</v>
       </c>
       <c r="L50" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.2">
@@ -2998,23 +3044,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/sweater_white.jpg</v>
       </c>
       <c r="B51" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C51" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D51" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E51" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F51" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G51">
         <f t="shared" ca="1" si="6"/>
-        <v>1899</v>
+        <v>3199</v>
       </c>
       <c r="H51">
         <f t="shared" si="2"/>
@@ -3031,7 +3077,7 @@
         <v>1</v>
       </c>
       <c r="L51" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
@@ -3040,23 +3086,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/sweatshirt_bright.jpg</v>
       </c>
       <c r="B52" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C52" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D52" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E52" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F52" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G52">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>2299</v>
       </c>
       <c r="H52">
         <f t="shared" si="2"/>
@@ -3073,7 +3119,7 @@
         <v>1</v>
       </c>
       <c r="L52" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.2">
@@ -3082,23 +3128,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/sweatshirt_pastel.jpg</v>
       </c>
       <c r="B53" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C53" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D53" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E53" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F53" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G53">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>4099</v>
       </c>
       <c r="H53">
         <f t="shared" si="2"/>
@@ -3115,7 +3161,7 @@
         <v>1</v>
       </c>
       <c r="L53" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.2">
@@ -3124,30 +3170,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/peplum top- yellow.avif</v>
       </c>
       <c r="B54" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C54" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D54" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E54" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F54" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G54">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>1099</v>
       </c>
       <c r="H54">
         <f t="shared" si="2"/>
         <v>1054</v>
       </c>
       <c r="I54" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J54">
         <v>5</v>
@@ -3156,7 +3202,7 @@
         <v>1</v>
       </c>
       <c r="L54" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
@@ -3165,30 +3211,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/black dress.avif</v>
       </c>
       <c r="B55" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D55" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E55" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F55" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G55">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>899</v>
       </c>
       <c r="H55">
         <f t="shared" si="2"/>
         <v>1055</v>
       </c>
       <c r="I55" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J55">
         <v>5</v>
@@ -3197,7 +3243,7 @@
         <v>1</v>
       </c>
       <c r="L55" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.2">
@@ -3206,30 +3252,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/black graphic tee.jpeg</v>
       </c>
       <c r="B56" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C56" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D56" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E56" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F56" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G56">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>2799</v>
       </c>
       <c r="H56">
         <f t="shared" si="2"/>
         <v>1056</v>
       </c>
       <c r="I56" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J56">
         <v>5</v>
@@ -3238,7 +3284,7 @@
         <v>1</v>
       </c>
       <c r="L56" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.2">
@@ -3247,30 +3293,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/black mini dress.avif</v>
       </c>
       <c r="B57" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C57" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D57" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E57" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F57" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G57">
         <f t="shared" ca="1" si="6"/>
-        <v>3499</v>
+        <v>3899</v>
       </c>
       <c r="H57">
         <f t="shared" si="2"/>
         <v>1057</v>
       </c>
       <c r="I57" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J57">
         <v>5</v>
@@ -3279,7 +3325,7 @@
         <v>1</v>
       </c>
       <c r="L57" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
@@ -3288,30 +3334,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blouse.avif</v>
       </c>
       <c r="B58" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C58" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D58" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E58" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F58" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G58">
         <f t="shared" ca="1" si="6"/>
-        <v>4499</v>
+        <v>1599</v>
       </c>
       <c r="H58">
         <f t="shared" si="2"/>
         <v>1058</v>
       </c>
       <c r="I58" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J58">
         <v>5</v>
@@ -3320,7 +3366,7 @@
         <v>1</v>
       </c>
       <c r="L58" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
@@ -3329,30 +3375,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue dress.avif</v>
       </c>
       <c r="B59" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C59" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D59" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E59" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F59" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G59">
         <f t="shared" ca="1" si="6"/>
-        <v>1299</v>
+        <v>3499</v>
       </c>
       <c r="H59">
         <f t="shared" si="2"/>
         <v>1059</v>
       </c>
       <c r="I59" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J59">
         <v>5</v>
@@ -3361,39 +3407,39 @@
         <v>1</v>
       </c>
       <c r="L59" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A60" t="str">
+        <f t="shared" si="4"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue jeans.avif</v>
+      </c>
+      <c r="B60" t="s">
+        <v>66</v>
+      </c>
+      <c r="C60" t="s">
+        <v>141</v>
+      </c>
+      <c r="D60" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A60" t="str">
-        <f t="shared" si="4"/>
-        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue jeans.avif</v>
-      </c>
-      <c r="B60" t="s">
-        <v>68</v>
-      </c>
-      <c r="C60" t="s">
-        <v>143</v>
-      </c>
-      <c r="D60" t="s">
-        <v>95</v>
-      </c>
       <c r="E60" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F60" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G60">
         <f t="shared" ca="1" si="6"/>
-        <v>2399</v>
+        <v>899</v>
       </c>
       <c r="H60">
         <f t="shared" si="2"/>
         <v>1060</v>
       </c>
       <c r="I60" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="J60">
         <v>3</v>
@@ -3402,7 +3448,7 @@
         <v>1</v>
       </c>
       <c r="L60" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.2">
@@ -3411,19 +3457,19 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/bodycon dress-blue.avif</v>
       </c>
       <c r="B61" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C61" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D61" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E61" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F61" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G61">
         <f t="shared" ca="1" si="6"/>
@@ -3434,7 +3480,7 @@
         <v>1061</v>
       </c>
       <c r="I61" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J61">
         <v>3</v>
@@ -3443,7 +3489,7 @@
         <v>1</v>
       </c>
       <c r="L61" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.2">
@@ -3452,30 +3498,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/brown blazer.avif</v>
       </c>
       <c r="B62" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C62" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D62" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E62" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F62" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G62">
         <f t="shared" ca="1" si="6"/>
-        <v>4299</v>
+        <v>2799</v>
       </c>
       <c r="H62">
         <f t="shared" si="2"/>
         <v>1062</v>
       </c>
       <c r="I62" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J62">
         <v>3</v>
@@ -3484,7 +3530,7 @@
         <v>1</v>
       </c>
       <c r="L62" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.2">
@@ -3493,30 +3539,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/brown dress.avif</v>
       </c>
       <c r="B63" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C63" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D63" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E63" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F63" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G63">
         <f t="shared" ca="1" si="6"/>
-        <v>4299</v>
+        <v>1299</v>
       </c>
       <c r="H63">
         <f t="shared" si="2"/>
         <v>1063</v>
       </c>
       <c r="I63" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J63">
         <v>3</v>
@@ -3525,39 +3571,39 @@
         <v>1</v>
       </c>
       <c r="L63" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A64" t="str">
+        <f t="shared" si="4"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Cargo pants.avif</v>
+      </c>
+      <c r="B64" t="s">
+        <v>70</v>
+      </c>
+      <c r="C64" t="s">
+        <v>151</v>
+      </c>
+      <c r="D64" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A64" t="str">
-        <f t="shared" si="4"/>
-        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Cargo pants.avif</v>
-      </c>
-      <c r="B64" t="s">
-        <v>72</v>
-      </c>
-      <c r="C64" t="s">
-        <v>153</v>
-      </c>
-      <c r="D64" t="s">
-        <v>95</v>
-      </c>
       <c r="E64" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F64" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G64">
         <f t="shared" ca="1" si="6"/>
-        <v>2099</v>
+        <v>2899</v>
       </c>
       <c r="H64">
         <f t="shared" si="2"/>
         <v>1064</v>
       </c>
       <c r="I64" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J64">
         <v>3</v>
@@ -3566,39 +3612,39 @@
         <v>1</v>
       </c>
       <c r="L64" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A65" t="str">
+        <f t="shared" si="4"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/cream palazo.avif</v>
+      </c>
+      <c r="B65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C65" t="s">
+        <v>151</v>
+      </c>
+      <c r="D65" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A65" t="str">
-        <f t="shared" si="4"/>
-        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/cream palazo.avif</v>
-      </c>
-      <c r="B65" t="s">
-        <v>73</v>
-      </c>
-      <c r="C65" t="s">
-        <v>153</v>
-      </c>
-      <c r="D65" t="s">
-        <v>95</v>
-      </c>
       <c r="E65" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F65" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G65">
         <f t="shared" ca="1" si="6"/>
-        <v>4899</v>
+        <v>4199</v>
       </c>
       <c r="H65">
         <f t="shared" si="2"/>
         <v>1065</v>
       </c>
       <c r="I65" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J65">
         <v>3</v>
@@ -3607,7 +3653,7 @@
         <v>1</v>
       </c>
       <c r="L65" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.2">
@@ -3616,30 +3662,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/croptop.jpeg</v>
       </c>
       <c r="B66" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C66" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D66" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E66" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F66" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G66">
         <f t="shared" ca="1" si="6"/>
-        <v>3499</v>
+        <v>1399</v>
       </c>
       <c r="H66">
         <f t="shared" si="2"/>
         <v>1066</v>
       </c>
       <c r="I66" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J66">
         <v>3</v>
@@ -3648,39 +3694,39 @@
         <v>1</v>
       </c>
       <c r="L66" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A67" t="str">
+        <f t="shared" si="4"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Culottes.avif</v>
+      </c>
+      <c r="B67" t="s">
+        <v>73</v>
+      </c>
+      <c r="C67" t="s">
+        <v>151</v>
+      </c>
+      <c r="D67" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A67" t="str">
-        <f t="shared" si="4"/>
-        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Culottes.avif</v>
-      </c>
-      <c r="B67" t="s">
-        <v>75</v>
-      </c>
-      <c r="C67" t="s">
-        <v>153</v>
-      </c>
-      <c r="D67" t="s">
-        <v>95</v>
-      </c>
       <c r="E67" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F67" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G67">
         <f t="shared" ca="1" si="6"/>
-        <v>1399</v>
+        <v>1899</v>
       </c>
       <c r="H67">
         <f t="shared" ref="H67:H79" si="7">ROW()+1000</f>
         <v>1067</v>
       </c>
       <c r="I67" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J67">
         <v>3</v>
@@ -3689,7 +3735,7 @@
         <v>1</v>
       </c>
       <c r="L67" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.2">
@@ -3698,30 +3744,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/halterneck top.avif</v>
       </c>
       <c r="B68" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C68" t="s">
+        <v>115</v>
+      </c>
+      <c r="D68" t="s">
+        <v>92</v>
+      </c>
+      <c r="E68" t="s">
+        <v>104</v>
+      </c>
+      <c r="F68" t="s">
         <v>117</v>
       </c>
-      <c r="D68" t="s">
-        <v>94</v>
-      </c>
-      <c r="E68" t="s">
-        <v>106</v>
-      </c>
-      <c r="F68" t="s">
-        <v>119</v>
-      </c>
       <c r="G68">
         <f t="shared" ca="1" si="6"/>
-        <v>1799</v>
+        <v>3299</v>
       </c>
       <c r="H68">
         <f t="shared" si="7"/>
         <v>1068</v>
       </c>
       <c r="I68" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J68">
         <v>3</v>
@@ -3730,28 +3776,28 @@
         <v>1</v>
       </c>
       <c r="L68" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A69" t="str">
+        <f t="shared" si="4"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Jeggings.avif</v>
+      </c>
+      <c r="B69" t="s">
+        <v>75</v>
+      </c>
+      <c r="C69" t="s">
+        <v>141</v>
+      </c>
+      <c r="D69" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A69" t="str">
-        <f t="shared" si="4"/>
-        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Jeggings.avif</v>
-      </c>
-      <c r="B69" t="s">
-        <v>77</v>
-      </c>
-      <c r="C69" t="s">
-        <v>143</v>
-      </c>
-      <c r="D69" t="s">
-        <v>95</v>
-      </c>
       <c r="E69" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F69" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G69">
         <f t="shared" ca="1" si="6"/>
@@ -3762,7 +3808,7 @@
         <v>1069</v>
       </c>
       <c r="I69" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J69">
         <v>3</v>
@@ -3771,39 +3817,39 @@
         <v>1</v>
       </c>
       <c r="L69" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A70" t="str">
+        <f t="shared" si="4"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Leggings.avif</v>
+      </c>
+      <c r="B70" t="s">
+        <v>76</v>
+      </c>
+      <c r="C70" t="s">
+        <v>112</v>
+      </c>
+      <c r="D70" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A70" t="str">
-        <f t="shared" si="4"/>
-        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/Leggings.avif</v>
-      </c>
-      <c r="B70" t="s">
-        <v>78</v>
-      </c>
-      <c r="C70" t="s">
-        <v>114</v>
-      </c>
-      <c r="D70" t="s">
-        <v>95</v>
-      </c>
       <c r="E70" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F70" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G70">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>4899</v>
       </c>
       <c r="H70">
         <f t="shared" si="7"/>
         <v>1070</v>
       </c>
       <c r="I70" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J70">
         <v>3</v>
@@ -3812,7 +3858,7 @@
         <v>1</v>
       </c>
       <c r="L70" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.2">
@@ -3821,30 +3867,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/off shoulder-brown.avif</v>
       </c>
       <c r="B71" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C71" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D71" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E71" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F71" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G71">
         <f t="shared" ca="1" si="6"/>
-        <v>3899</v>
+        <v>4399</v>
       </c>
       <c r="H71">
         <f t="shared" si="7"/>
         <v>1071</v>
       </c>
       <c r="I71" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J71">
         <v>3</v>
@@ -3853,39 +3899,39 @@
         <v>1</v>
       </c>
       <c r="L71" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A72" t="str">
-        <f t="shared" ref="A72:A83" si="8">"https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/" &amp; B72</f>
+        <f t="shared" ref="A72:A96" si="8">"https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/" &amp; B72</f>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink cardigan.avif</v>
       </c>
       <c r="B72" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C72" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D72" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E72" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F72" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G72">
         <f t="shared" ca="1" si="6"/>
-        <v>3199</v>
+        <v>3299</v>
       </c>
       <c r="H72">
         <f t="shared" si="7"/>
         <v>1072</v>
       </c>
       <c r="I72" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J72">
         <v>3</v>
@@ -3894,39 +3940,39 @@
         <v>1</v>
       </c>
       <c r="L72" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="str">
         <f t="shared" si="8"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink denim skirt.avif</v>
       </c>
       <c r="B73" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C73" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D73" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E73" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F73" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G73">
         <f t="shared" ca="1" si="6"/>
-        <v>2599</v>
+        <v>3699</v>
       </c>
       <c r="H73">
         <f t="shared" si="7"/>
         <v>1073</v>
       </c>
       <c r="I73" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J73">
         <v>3</v>
@@ -3935,7 +3981,7 @@
         <v>1</v>
       </c>
       <c r="L73" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.2">
@@ -3944,30 +3990,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink hoodie.avif</v>
       </c>
       <c r="B74" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C74" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D74" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E74" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F74" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G74">
         <f t="shared" ca="1" si="6"/>
-        <v>3199</v>
+        <v>2099</v>
       </c>
       <c r="H74">
         <f t="shared" si="7"/>
         <v>1074</v>
       </c>
       <c r="I74" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J74">
         <v>3</v>
@@ -3976,7 +4022,7 @@
         <v>1</v>
       </c>
       <c r="L74" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.2">
@@ -3985,30 +4031,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/shirt-white.avif</v>
       </c>
       <c r="B75" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C75" t="s">
+        <v>115</v>
+      </c>
+      <c r="D75" t="s">
+        <v>92</v>
+      </c>
+      <c r="E75" t="s">
+        <v>97</v>
+      </c>
+      <c r="F75" t="s">
         <v>117</v>
       </c>
-      <c r="D75" t="s">
-        <v>94</v>
-      </c>
-      <c r="E75" t="s">
-        <v>99</v>
-      </c>
-      <c r="F75" t="s">
-        <v>119</v>
-      </c>
       <c r="G75">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>4599</v>
       </c>
       <c r="H75">
         <f t="shared" si="7"/>
         <v>1075</v>
       </c>
       <c r="I75" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J75">
         <v>6</v>
@@ -4017,7 +4063,7 @@
         <v>1</v>
       </c>
       <c r="L75" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.2">
@@ -4026,30 +4072,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/tanktop.jpeg</v>
       </c>
       <c r="B76" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C76" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D76" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E76" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F76" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G76">
         <f t="shared" ca="1" si="6"/>
-        <v>1299</v>
+        <v>2199</v>
       </c>
       <c r="H76">
         <f t="shared" si="7"/>
         <v>1076</v>
       </c>
       <c r="I76" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J76">
         <v>6</v>
@@ -4058,39 +4104,39 @@
         <v>1</v>
       </c>
       <c r="L76" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="str">
         <f t="shared" si="8"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/trouser-black.avif</v>
       </c>
       <c r="B77" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C77" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D77" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E77" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F77" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G77">
         <f t="shared" ca="1" si="6"/>
-        <v>1999</v>
+        <v>2499</v>
       </c>
       <c r="H77">
         <f t="shared" si="7"/>
         <v>1077</v>
       </c>
       <c r="I77" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J77">
         <v>6</v>
@@ -4099,7 +4145,7 @@
         <v>1</v>
       </c>
       <c r="L77" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
@@ -4108,30 +4154,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/tube top.avif</v>
       </c>
       <c r="B78" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C78" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D78" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E78" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F78" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G78">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>4399</v>
       </c>
       <c r="H78">
         <f t="shared" si="7"/>
         <v>1078</v>
       </c>
       <c r="I78" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J78">
         <v>6</v>
@@ -4140,7 +4186,7 @@
         <v>1</v>
       </c>
       <c r="L78" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
@@ -4149,30 +4195,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/tunic dress.avif</v>
       </c>
       <c r="B79" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C79" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D79" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E79" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F79" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G79">
-        <f t="shared" ref="G79:G83" ca="1" si="9">RANDBETWEEN(7,49)*100+99</f>
-        <v>4399</v>
+        <f t="shared" ref="G79:G96" ca="1" si="9">RANDBETWEEN(7,49)*100+99</f>
+        <v>1199</v>
       </c>
       <c r="H79">
         <f t="shared" si="7"/>
         <v>1079</v>
       </c>
       <c r="I79" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J79">
         <v>6</v>
@@ -4181,39 +4227,39 @@
         <v>1</v>
       </c>
       <c r="L79" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" t="str">
         <f t="shared" si="8"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/white denim shorts.avif</v>
       </c>
       <c r="B80" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C80" t="s">
+        <v>115</v>
+      </c>
+      <c r="D80" t="s">
+        <v>93</v>
+      </c>
+      <c r="E80" t="s">
+        <v>94</v>
+      </c>
+      <c r="F80" t="s">
         <v>117</v>
-      </c>
-      <c r="D80" t="s">
-        <v>95</v>
-      </c>
-      <c r="E80" t="s">
-        <v>96</v>
-      </c>
-      <c r="F80" t="s">
-        <v>119</v>
       </c>
       <c r="G80">
         <f t="shared" ca="1" si="9"/>
-        <v>4399</v>
+        <v>2799</v>
       </c>
       <c r="H80">
         <f>ROW()+1000</f>
         <v>1080</v>
       </c>
       <c r="I80" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J80">
         <v>6</v>
@@ -4222,7 +4268,7 @@
         <v>1</v>
       </c>
       <c r="L80" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.2">
@@ -4231,30 +4277,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/white shirt dress.avif</v>
       </c>
       <c r="B81" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C81" t="s">
+        <v>115</v>
+      </c>
+      <c r="D81" t="s">
+        <v>92</v>
+      </c>
+      <c r="E81" t="s">
+        <v>111</v>
+      </c>
+      <c r="F81" t="s">
         <v>117</v>
-      </c>
-      <c r="D81" t="s">
-        <v>94</v>
-      </c>
-      <c r="E81" t="s">
-        <v>113</v>
-      </c>
-      <c r="F81" t="s">
-        <v>119</v>
       </c>
       <c r="G81">
         <f t="shared" ca="1" si="9"/>
-        <v>1799</v>
+        <v>4799</v>
       </c>
       <c r="H81">
-        <f t="shared" ref="H81:H83" si="10">ROW()+1000</f>
+        <f t="shared" ref="H81:H96" si="10">ROW()+1000</f>
         <v>1081</v>
       </c>
       <c r="I81" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J81">
         <v>6</v>
@@ -4263,7 +4309,7 @@
         <v>1</v>
       </c>
       <c r="L81" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.2">
@@ -4272,30 +4318,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/white strappy dress.avif</v>
       </c>
       <c r="B82" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C82" t="s">
+        <v>115</v>
+      </c>
+      <c r="D82" t="s">
+        <v>92</v>
+      </c>
+      <c r="E82" t="s">
+        <v>103</v>
+      </c>
+      <c r="F82" t="s">
         <v>117</v>
-      </c>
-      <c r="D82" t="s">
-        <v>94</v>
-      </c>
-      <c r="E82" t="s">
-        <v>105</v>
-      </c>
-      <c r="F82" t="s">
-        <v>119</v>
       </c>
       <c r="G82">
         <f t="shared" ca="1" si="9"/>
-        <v>3999</v>
+        <v>1299</v>
       </c>
       <c r="H82">
         <f t="shared" si="10"/>
         <v>1082</v>
       </c>
       <c r="I82" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="J82">
         <v>6</v>
@@ -4304,7 +4350,7 @@
         <v>1</v>
       </c>
       <c r="L82" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.2">
@@ -4313,30 +4359,30 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/white tee.jpeg</v>
       </c>
       <c r="B83" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C83" t="s">
+        <v>115</v>
+      </c>
+      <c r="D83" t="s">
+        <v>92</v>
+      </c>
+      <c r="E83" t="s">
+        <v>103</v>
+      </c>
+      <c r="F83" t="s">
         <v>117</v>
-      </c>
-      <c r="D83" t="s">
-        <v>94</v>
-      </c>
-      <c r="E83" t="s">
-        <v>105</v>
-      </c>
-      <c r="F83" t="s">
-        <v>119</v>
       </c>
       <c r="G83">
         <f t="shared" ca="1" si="9"/>
-        <v>4599</v>
+        <v>3899</v>
       </c>
       <c r="H83">
         <f t="shared" si="10"/>
         <v>1083</v>
       </c>
       <c r="I83" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="J83">
         <v>6</v>
@@ -4345,11 +4391,550 @@
         <v>1</v>
       </c>
       <c r="L83" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A84" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/black formal pants.avif</v>
+      </c>
+      <c r="B84" t="s">
+        <v>163</v>
+      </c>
+      <c r="C84" t="s">
+        <v>137</v>
+      </c>
+      <c r="D84" t="s">
         <v>93</v>
       </c>
+      <c r="E84" t="s">
+        <v>177</v>
+      </c>
+      <c r="F84" t="s">
+        <v>112</v>
+      </c>
+      <c r="G84">
+        <f t="shared" ca="1" si="9"/>
+        <v>1199</v>
+      </c>
+      <c r="H84">
+        <f t="shared" si="10"/>
+        <v>1084</v>
+      </c>
+      <c r="I84" t="s">
+        <v>175</v>
+      </c>
+      <c r="J84">
+        <v>6</v>
+      </c>
+      <c r="K84" t="b">
+        <v>1</v>
+      </c>
+      <c r="L84" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A85" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue croptop.avif</v>
+      </c>
+      <c r="B85" t="s">
+        <v>164</v>
+      </c>
+      <c r="C85" t="s">
+        <v>176</v>
+      </c>
+      <c r="D85" t="s">
+        <v>92</v>
+      </c>
+      <c r="E85" t="s">
+        <v>103</v>
+      </c>
+      <c r="F85" t="s">
+        <v>114</v>
+      </c>
+      <c r="G85">
+        <f t="shared" ca="1" si="9"/>
+        <v>2199</v>
+      </c>
+      <c r="H85">
+        <f t="shared" si="10"/>
+        <v>1085</v>
+      </c>
+      <c r="I85" t="s">
+        <v>92</v>
+      </c>
+      <c r="J85">
+        <v>6</v>
+      </c>
+      <c r="K85" t="b">
+        <v>1</v>
+      </c>
+      <c r="L85" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A86" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue jeans.avif</v>
+      </c>
+      <c r="B86" t="s">
+        <v>66</v>
+      </c>
+      <c r="C86" t="s">
+        <v>141</v>
+      </c>
+      <c r="D86" t="s">
+        <v>93</v>
+      </c>
+      <c r="E86" t="s">
+        <v>99</v>
+      </c>
+      <c r="F86" t="s">
+        <v>116</v>
+      </c>
+      <c r="G86">
+        <f t="shared" ca="1" si="9"/>
+        <v>799</v>
+      </c>
+      <c r="H86">
+        <f t="shared" si="10"/>
+        <v>1086</v>
+      </c>
+      <c r="I86" t="s">
+        <v>93</v>
+      </c>
+      <c r="J86">
+        <v>6</v>
+      </c>
+      <c r="K86" t="b">
+        <v>1</v>
+      </c>
+      <c r="L86" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A87" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/halter neck sequined.avif</v>
+      </c>
+      <c r="B87" t="s">
+        <v>165</v>
+      </c>
+      <c r="C87" t="s">
+        <v>131</v>
+      </c>
+      <c r="D87" t="s">
+        <v>92</v>
+      </c>
+      <c r="E87" t="s">
+        <v>110</v>
+      </c>
+      <c r="F87" t="s">
+        <v>113</v>
+      </c>
+      <c r="G87">
+        <f t="shared" ca="1" si="9"/>
+        <v>999</v>
+      </c>
+      <c r="H87">
+        <f t="shared" si="10"/>
+        <v>1087</v>
+      </c>
+      <c r="I87" t="s">
+        <v>92</v>
+      </c>
+      <c r="J87">
+        <v>6</v>
+      </c>
+      <c r="K87" t="b">
+        <v>1</v>
+      </c>
+      <c r="L87" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A88" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/khaki green formal trouser.avif</v>
+      </c>
+      <c r="B88" t="s">
+        <v>166</v>
+      </c>
+      <c r="C88" t="s">
+        <v>143</v>
+      </c>
+      <c r="D88" t="s">
+        <v>93</v>
+      </c>
+      <c r="E88" t="s">
+        <v>97</v>
+      </c>
+      <c r="F88" t="s">
+        <v>113</v>
+      </c>
+      <c r="G88">
+        <f t="shared" ca="1" si="9"/>
+        <v>1499</v>
+      </c>
+      <c r="H88">
+        <f t="shared" si="10"/>
+        <v>1088</v>
+      </c>
+      <c r="I88" t="s">
+        <v>175</v>
+      </c>
+      <c r="J88">
+        <v>6</v>
+      </c>
+      <c r="K88" t="b">
+        <v>1</v>
+      </c>
+      <c r="L88" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A89" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/light blue full sleeve shirt.avif</v>
+      </c>
+      <c r="B89" t="s">
+        <v>167</v>
+      </c>
+      <c r="C89" t="s">
+        <v>142</v>
+      </c>
+      <c r="D89" t="s">
+        <v>92</v>
+      </c>
+      <c r="E89" t="s">
+        <v>157</v>
+      </c>
+      <c r="F89" t="s">
+        <v>114</v>
+      </c>
+      <c r="G89">
+        <f t="shared" ca="1" si="9"/>
+        <v>2299</v>
+      </c>
+      <c r="H89">
+        <f t="shared" si="10"/>
+        <v>1089</v>
+      </c>
+      <c r="I89" t="s">
+        <v>92</v>
+      </c>
+      <c r="J89">
+        <v>6</v>
+      </c>
+      <c r="K89" t="b">
+        <v>1</v>
+      </c>
+      <c r="L89" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A90" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink flounced blouse.avif</v>
+      </c>
+      <c r="B90" t="s">
+        <v>168</v>
+      </c>
+      <c r="C90" t="s">
+        <v>154</v>
+      </c>
+      <c r="D90" t="s">
+        <v>92</v>
+      </c>
+      <c r="E90" t="s">
+        <v>103</v>
+      </c>
+      <c r="F90" t="s">
+        <v>114</v>
+      </c>
+      <c r="G90">
+        <f t="shared" ca="1" si="9"/>
+        <v>1899</v>
+      </c>
+      <c r="H90">
+        <f t="shared" si="10"/>
+        <v>1090</v>
+      </c>
+      <c r="I90" t="s">
+        <v>92</v>
+      </c>
+      <c r="J90">
+        <v>6</v>
+      </c>
+      <c r="K90" t="b">
+        <v>1</v>
+      </c>
+      <c r="L90" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="91" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A91" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink tank top.avif</v>
+      </c>
+      <c r="B91" t="s">
+        <v>169</v>
+      </c>
+      <c r="C91" t="s">
+        <v>154</v>
+      </c>
+      <c r="D91" t="s">
+        <v>92</v>
+      </c>
+      <c r="E91" t="s">
+        <v>103</v>
+      </c>
+      <c r="F91" t="s">
+        <v>114</v>
+      </c>
+      <c r="G91">
+        <f t="shared" ca="1" si="9"/>
+        <v>2999</v>
+      </c>
+      <c r="H91">
+        <f t="shared" si="10"/>
+        <v>1091</v>
+      </c>
+      <c r="I91" t="s">
+        <v>92</v>
+      </c>
+      <c r="J91">
+        <v>6</v>
+      </c>
+      <c r="K91" t="b">
+        <v>1</v>
+      </c>
+      <c r="L91" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A92" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red fine knit.jpeg</v>
+      </c>
+      <c r="B92" t="s">
+        <v>170</v>
+      </c>
+      <c r="C92" t="s">
+        <v>144</v>
+      </c>
+      <c r="D92" t="s">
+        <v>92</v>
+      </c>
+      <c r="E92" t="s">
+        <v>103</v>
+      </c>
+      <c r="F92" t="s">
+        <v>117</v>
+      </c>
+      <c r="G92">
+        <f t="shared" ca="1" si="9"/>
+        <v>1099</v>
+      </c>
+      <c r="H92">
+        <f t="shared" si="10"/>
+        <v>1092</v>
+      </c>
+      <c r="I92" t="s">
+        <v>92</v>
+      </c>
+      <c r="J92">
+        <v>6</v>
+      </c>
+      <c r="K92" t="b">
+        <v>1</v>
+      </c>
+      <c r="L92" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A93" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red halter.avif</v>
+      </c>
+      <c r="B93" t="s">
+        <v>171</v>
+      </c>
+      <c r="C93" t="s">
+        <v>144</v>
+      </c>
+      <c r="D93" t="s">
+        <v>92</v>
+      </c>
+      <c r="E93" t="s">
+        <v>103</v>
+      </c>
+      <c r="F93" t="s">
+        <v>117</v>
+      </c>
+      <c r="G93">
+        <f t="shared" ca="1" si="9"/>
+        <v>2399</v>
+      </c>
+      <c r="H93">
+        <f t="shared" si="10"/>
+        <v>1093</v>
+      </c>
+      <c r="I93" t="s">
+        <v>92</v>
+      </c>
+      <c r="J93">
+        <v>6</v>
+      </c>
+      <c r="K93" t="b">
+        <v>1</v>
+      </c>
+      <c r="L93" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A94" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red peplum.avif</v>
+      </c>
+      <c r="B94" t="s">
+        <v>172</v>
+      </c>
+      <c r="C94" t="s">
+        <v>144</v>
+      </c>
+      <c r="D94" t="s">
+        <v>92</v>
+      </c>
+      <c r="E94" t="s">
+        <v>103</v>
+      </c>
+      <c r="F94" t="s">
+        <v>117</v>
+      </c>
+      <c r="G94">
+        <f t="shared" ca="1" si="9"/>
+        <v>2199</v>
+      </c>
+      <c r="H94">
+        <f t="shared" si="10"/>
+        <v>1094</v>
+      </c>
+      <c r="I94" t="s">
+        <v>92</v>
+      </c>
+      <c r="J94">
+        <v>6</v>
+      </c>
+      <c r="K94" t="b">
+        <v>1</v>
+      </c>
+      <c r="L94" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A95" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/white formal pants.avif</v>
+      </c>
+      <c r="B95" t="s">
+        <v>173</v>
+      </c>
+      <c r="C95" t="s">
+        <v>115</v>
+      </c>
+      <c r="D95" t="s">
+        <v>93</v>
+      </c>
+      <c r="E95" t="s">
+        <v>177</v>
+      </c>
+      <c r="F95" t="s">
+        <v>115</v>
+      </c>
+      <c r="G95">
+        <f t="shared" ca="1" si="9"/>
+        <v>1399</v>
+      </c>
+      <c r="H95">
+        <f t="shared" si="10"/>
+        <v>1095</v>
+      </c>
+      <c r="I95" t="s">
+        <v>175</v>
+      </c>
+      <c r="J95">
+        <v>6</v>
+      </c>
+      <c r="K95" t="b">
+        <v>1</v>
+      </c>
+      <c r="L95" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="96" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A96" t="str">
+        <f t="shared" si="8"/>
+        <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/yellow top.avif</v>
+      </c>
+      <c r="B96" t="s">
+        <v>174</v>
+      </c>
+      <c r="C96" t="s">
+        <v>147</v>
+      </c>
+      <c r="D96" t="s">
+        <v>92</v>
+      </c>
+      <c r="E96" t="s">
+        <v>103</v>
+      </c>
+      <c r="F96" t="s">
+        <v>117</v>
+      </c>
+      <c r="G96">
+        <f t="shared" ca="1" si="9"/>
+        <v>3699</v>
+      </c>
+      <c r="H96">
+        <f t="shared" si="10"/>
+        <v>1096</v>
+      </c>
+      <c r="I96" t="s">
+        <v>92</v>
+      </c>
+      <c r="J96">
+        <v>6</v>
+      </c>
+      <c r="K96" t="b">
+        <v>1</v>
+      </c>
+      <c r="L96" t="s">
+        <v>91</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{BC477210-8802-4647-A9A0-82022E3B188B}"/>
+  <autoFilter ref="A1:K83" xr:uid="{BC477210-8802-4647-A9A0-82022E3B188B}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="top"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
updated excel data structure
</commit_message>
<xml_diff>
--- a/styleshop.xlsx
+++ b/styleshop.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aryanbhandari/aryancoding/styleshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884DC111-4A38-3E42-8F7A-51285E6974E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF82B83-CED5-9D41-8A47-8AA37542C4C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{296FE156-ABE8-A143-BE54-67E50949700F}"/>
   </bookViews>
@@ -527,9 +527,6 @@
     <t>formalshirt_white.jpg</t>
   </si>
   <si>
-    <t xml:space="preserve">gender = male </t>
-  </si>
-  <si>
     <t>black formal pants.avif</t>
   </si>
   <si>
@@ -573,6 +570,9 @@
   </si>
   <si>
     <t xml:space="preserve">formal </t>
+  </si>
+  <si>
+    <t xml:space="preserve">gender  </t>
   </si>
 </sst>
 </file>
@@ -990,7 +990,7 @@
         <v>6</v>
       </c>
       <c r="L1" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="G2">
         <f ca="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>1999</v>
+        <v>1099</v>
       </c>
       <c r="H2">
         <f>ROW()+1000</f>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G6" ca="1" si="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>1899</v>
+        <v>999</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H66" si="2">ROW()+1000</f>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="G4">
         <f t="shared" ca="1" si="1"/>
-        <v>1899</v>
+        <v>899</v>
       </c>
       <c r="H4">
         <f t="shared" si="2"/>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G5">
         <f t="shared" ca="1" si="1"/>
-        <v>1699</v>
+        <v>1599</v>
       </c>
       <c r="H5">
         <f t="shared" si="2"/>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="G6">
         <f t="shared" ca="1" si="1"/>
-        <v>1399</v>
+        <v>1699</v>
       </c>
       <c r="H6">
         <f t="shared" si="2"/>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="G7">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
-        <v>3299</v>
+        <v>2099</v>
       </c>
       <c r="H7">
         <f t="shared" si="2"/>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G8">
         <f t="shared" ref="G8:G13" ca="1" si="5">RANDBETWEEN(19,49)*100+99</f>
-        <v>3099</v>
+        <v>2799</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="5"/>
-        <v>4699</v>
+        <v>3499</v>
       </c>
       <c r="H9">
         <f t="shared" si="2"/>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="5"/>
-        <v>2899</v>
+        <v>2499</v>
       </c>
       <c r="H10">
         <f t="shared" si="2"/>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="5"/>
-        <v>2699</v>
+        <v>4099</v>
       </c>
       <c r="H11">
         <f t="shared" si="2"/>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="G12">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
-        <v>2499</v>
+        <v>4399</v>
       </c>
       <c r="H12">
         <f t="shared" si="2"/>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="5"/>
-        <v>3499</v>
+        <v>4399</v>
       </c>
       <c r="H13">
         <f t="shared" si="2"/>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="G14">
         <f ca="1">RANDBETWEEN(7,49)*100+99</f>
-        <v>2099</v>
+        <v>1799</v>
       </c>
       <c r="H14">
         <f t="shared" si="2"/>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="G15">
         <f t="shared" ref="G15:G78" ca="1" si="6">RANDBETWEEN(7,49)*100+99</f>
-        <v>3999</v>
+        <v>3599</v>
       </c>
       <c r="H15">
         <f t="shared" si="2"/>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>4899</v>
       </c>
       <c r="H16">
         <f t="shared" si="2"/>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="G17">
         <f t="shared" ca="1" si="6"/>
-        <v>3199</v>
+        <v>4699</v>
       </c>
       <c r="H17">
         <f t="shared" si="2"/>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="G18">
         <f t="shared" ca="1" si="6"/>
-        <v>1599</v>
+        <v>1699</v>
       </c>
       <c r="H18">
         <f t="shared" si="2"/>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="G19">
         <f t="shared" ca="1" si="6"/>
-        <v>4499</v>
+        <v>999</v>
       </c>
       <c r="H19">
         <f t="shared" si="2"/>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="G20">
         <f t="shared" ca="1" si="6"/>
-        <v>1599</v>
+        <v>1099</v>
       </c>
       <c r="H20">
         <f t="shared" si="2"/>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G21">
         <f t="shared" ca="1" si="6"/>
-        <v>4699</v>
+        <v>4999</v>
       </c>
       <c r="H21">
         <f t="shared" si="2"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="G22">
         <f t="shared" ca="1" si="6"/>
-        <v>1699</v>
+        <v>2499</v>
       </c>
       <c r="H22">
         <f t="shared" si="2"/>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="G23">
         <f t="shared" ca="1" si="6"/>
-        <v>3799</v>
+        <v>1499</v>
       </c>
       <c r="H23">
         <f t="shared" si="2"/>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="G24">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>1699</v>
       </c>
       <c r="H24">
         <f t="shared" si="2"/>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="G25">
         <f t="shared" ca="1" si="6"/>
-        <v>4999</v>
+        <v>4599</v>
       </c>
       <c r="H25">
         <f t="shared" si="2"/>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="G26">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>3899</v>
       </c>
       <c r="H26">
         <f t="shared" si="2"/>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="G27">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>3099</v>
       </c>
       <c r="H27">
         <f t="shared" si="2"/>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="G28">
         <f t="shared" ca="1" si="6"/>
-        <v>1199</v>
+        <v>2299</v>
       </c>
       <c r="H28">
         <f t="shared" si="2"/>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="G29">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>1699</v>
       </c>
       <c r="H29">
         <f t="shared" si="2"/>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="G30">
         <f t="shared" ca="1" si="6"/>
-        <v>2799</v>
+        <v>3699</v>
       </c>
       <c r="H30">
         <f t="shared" si="2"/>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="G31">
         <f t="shared" ca="1" si="6"/>
-        <v>2799</v>
+        <v>899</v>
       </c>
       <c r="H31">
         <f t="shared" si="2"/>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="G32">
         <f t="shared" ca="1" si="6"/>
-        <v>3399</v>
+        <v>899</v>
       </c>
       <c r="H32">
         <f t="shared" si="2"/>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="G33">
         <f t="shared" ca="1" si="6"/>
-        <v>2799</v>
+        <v>899</v>
       </c>
       <c r="H33">
         <f t="shared" si="2"/>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="G34">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>1699</v>
       </c>
       <c r="H34">
         <f t="shared" si="2"/>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="G35">
         <f t="shared" ca="1" si="6"/>
-        <v>3899</v>
+        <v>4799</v>
       </c>
       <c r="H35">
         <f t="shared" si="2"/>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="G37">
         <f t="shared" ca="1" si="6"/>
-        <v>999</v>
+        <v>799</v>
       </c>
       <c r="H37">
         <f t="shared" si="2"/>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="G38">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>3299</v>
       </c>
       <c r="H38">
         <f t="shared" si="2"/>
@@ -2563,7 +2563,7 @@
       </c>
       <c r="G39">
         <f t="shared" ca="1" si="6"/>
-        <v>2399</v>
+        <v>1499</v>
       </c>
       <c r="H39">
         <f t="shared" si="2"/>
@@ -2605,7 +2605,7 @@
       </c>
       <c r="G40">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>3699</v>
       </c>
       <c r="H40">
         <f t="shared" si="2"/>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="G41">
         <f t="shared" ca="1" si="6"/>
-        <v>999</v>
+        <v>4299</v>
       </c>
       <c r="H41">
         <f t="shared" si="2"/>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="G42">
         <f t="shared" ca="1" si="6"/>
-        <v>3599</v>
+        <v>4499</v>
       </c>
       <c r="H42">
         <f t="shared" si="2"/>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="G43">
         <f t="shared" ca="1" si="6"/>
-        <v>1899</v>
+        <v>4599</v>
       </c>
       <c r="H43">
         <f t="shared" si="2"/>
@@ -2769,7 +2769,7 @@
       </c>
       <c r="G44">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>2399</v>
       </c>
       <c r="H44">
         <f t="shared" si="2"/>
@@ -2852,7 +2852,7 @@
       </c>
       <c r="G46">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>3399</v>
       </c>
       <c r="H46">
         <f t="shared" si="2"/>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="G47">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>2799</v>
       </c>
       <c r="H47">
         <f t="shared" si="2"/>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="G48">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>1799</v>
       </c>
       <c r="H48">
         <f t="shared" si="2"/>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G49">
         <f t="shared" ca="1" si="6"/>
-        <v>3799</v>
+        <v>999</v>
       </c>
       <c r="H49">
         <f t="shared" si="2"/>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="G50">
         <f t="shared" ca="1" si="6"/>
-        <v>1399</v>
+        <v>3999</v>
       </c>
       <c r="H50">
         <f t="shared" si="2"/>
@@ -3060,7 +3060,7 @@
       </c>
       <c r="G51">
         <f t="shared" ca="1" si="6"/>
-        <v>3199</v>
+        <v>3099</v>
       </c>
       <c r="H51">
         <f t="shared" si="2"/>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="G52">
         <f t="shared" ca="1" si="6"/>
-        <v>2299</v>
+        <v>2899</v>
       </c>
       <c r="H52">
         <f t="shared" si="2"/>
@@ -3144,7 +3144,7 @@
       </c>
       <c r="G53">
         <f t="shared" ca="1" si="6"/>
-        <v>4099</v>
+        <v>4199</v>
       </c>
       <c r="H53">
         <f t="shared" si="2"/>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="G54">
         <f t="shared" ca="1" si="6"/>
-        <v>1099</v>
+        <v>2599</v>
       </c>
       <c r="H54">
         <f t="shared" si="2"/>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="G55">
         <f t="shared" ca="1" si="6"/>
-        <v>899</v>
+        <v>3999</v>
       </c>
       <c r="H55">
         <f t="shared" si="2"/>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="G56">
         <f t="shared" ca="1" si="6"/>
-        <v>2799</v>
+        <v>2499</v>
       </c>
       <c r="H56">
         <f t="shared" si="2"/>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="G57">
         <f t="shared" ca="1" si="6"/>
-        <v>3899</v>
+        <v>2899</v>
       </c>
       <c r="H57">
         <f t="shared" si="2"/>
@@ -3350,7 +3350,7 @@
       </c>
       <c r="G58">
         <f t="shared" ca="1" si="6"/>
-        <v>1599</v>
+        <v>1999</v>
       </c>
       <c r="H58">
         <f t="shared" si="2"/>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="G59">
         <f t="shared" ca="1" si="6"/>
-        <v>3499</v>
+        <v>2899</v>
       </c>
       <c r="H59">
         <f t="shared" si="2"/>
@@ -3432,7 +3432,7 @@
       </c>
       <c r="G60">
         <f t="shared" ca="1" si="6"/>
-        <v>899</v>
+        <v>2499</v>
       </c>
       <c r="H60">
         <f t="shared" si="2"/>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="G61">
         <f t="shared" ca="1" si="6"/>
-        <v>3899</v>
+        <v>2299</v>
       </c>
       <c r="H61">
         <f t="shared" si="2"/>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="G62">
         <f t="shared" ca="1" si="6"/>
-        <v>2799</v>
+        <v>1599</v>
       </c>
       <c r="H62">
         <f t="shared" si="2"/>
@@ -3555,7 +3555,7 @@
       </c>
       <c r="G63">
         <f t="shared" ca="1" si="6"/>
-        <v>1299</v>
+        <v>2799</v>
       </c>
       <c r="H63">
         <f t="shared" si="2"/>
@@ -3596,7 +3596,7 @@
       </c>
       <c r="G64">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>3899</v>
       </c>
       <c r="H64">
         <f t="shared" si="2"/>
@@ -3637,7 +3637,7 @@
       </c>
       <c r="G65">
         <f t="shared" ca="1" si="6"/>
-        <v>4199</v>
+        <v>899</v>
       </c>
       <c r="H65">
         <f t="shared" si="2"/>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="G66">
         <f t="shared" ca="1" si="6"/>
-        <v>1399</v>
+        <v>1999</v>
       </c>
       <c r="H66">
         <f t="shared" si="2"/>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="G67">
         <f t="shared" ca="1" si="6"/>
-        <v>1899</v>
+        <v>2899</v>
       </c>
       <c r="H67">
         <f t="shared" ref="H67:H79" si="7">ROW()+1000</f>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="G68">
         <f t="shared" ca="1" si="6"/>
-        <v>3299</v>
+        <v>3999</v>
       </c>
       <c r="H68">
         <f t="shared" si="7"/>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="G69">
         <f t="shared" ca="1" si="6"/>
-        <v>1699</v>
+        <v>1599</v>
       </c>
       <c r="H69">
         <f t="shared" si="7"/>
@@ -3842,7 +3842,7 @@
       </c>
       <c r="G70">
         <f t="shared" ca="1" si="6"/>
-        <v>4899</v>
+        <v>2399</v>
       </c>
       <c r="H70">
         <f t="shared" si="7"/>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="G71">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>2299</v>
       </c>
       <c r="H71">
         <f t="shared" si="7"/>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="G72">
         <f t="shared" ca="1" si="6"/>
-        <v>3299</v>
+        <v>799</v>
       </c>
       <c r="H72">
         <f t="shared" si="7"/>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="G73">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>2299</v>
       </c>
       <c r="H73">
         <f t="shared" si="7"/>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="G74">
         <f t="shared" ca="1" si="6"/>
-        <v>2099</v>
+        <v>1699</v>
       </c>
       <c r="H74">
         <f t="shared" si="7"/>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="G76">
         <f t="shared" ca="1" si="6"/>
-        <v>2199</v>
+        <v>1899</v>
       </c>
       <c r="H76">
         <f t="shared" si="7"/>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="G77">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>4199</v>
       </c>
       <c r="H77">
         <f t="shared" si="7"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="G78">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>4799</v>
       </c>
       <c r="H78">
         <f t="shared" si="7"/>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="G79">
         <f t="shared" ref="G79:G96" ca="1" si="9">RANDBETWEEN(7,49)*100+99</f>
-        <v>1199</v>
+        <v>1699</v>
       </c>
       <c r="H79">
         <f t="shared" si="7"/>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="G80">
         <f t="shared" ca="1" si="9"/>
-        <v>2799</v>
+        <v>2499</v>
       </c>
       <c r="H80">
         <f>ROW()+1000</f>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="G81">
         <f t="shared" ca="1" si="9"/>
-        <v>4799</v>
+        <v>2499</v>
       </c>
       <c r="H81">
         <f t="shared" ref="H81:H96" si="10">ROW()+1000</f>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="G82">
         <f t="shared" ca="1" si="9"/>
-        <v>1299</v>
+        <v>1899</v>
       </c>
       <c r="H82">
         <f t="shared" si="10"/>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="G83">
         <f t="shared" ca="1" si="9"/>
-        <v>3899</v>
+        <v>3399</v>
       </c>
       <c r="H83">
         <f t="shared" si="10"/>
@@ -4400,7 +4400,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/black formal pants.avif</v>
       </c>
       <c r="B84" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C84" t="s">
         <v>137</v>
@@ -4409,7 +4409,7 @@
         <v>93</v>
       </c>
       <c r="E84" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F84" t="s">
         <v>112</v>
@@ -4423,7 +4423,7 @@
         <v>1084</v>
       </c>
       <c r="I84" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J84">
         <v>6</v>
@@ -4441,10 +4441,10 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue croptop.avif</v>
       </c>
       <c r="B85" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C85" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D85" t="s">
         <v>92</v>
@@ -4457,7 +4457,7 @@
       </c>
       <c r="G85">
         <f t="shared" ca="1" si="9"/>
-        <v>2199</v>
+        <v>4999</v>
       </c>
       <c r="H85">
         <f t="shared" si="10"/>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="G86">
         <f t="shared" ca="1" si="9"/>
-        <v>799</v>
+        <v>1199</v>
       </c>
       <c r="H86">
         <f t="shared" si="10"/>
@@ -4523,7 +4523,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/halter neck sequined.avif</v>
       </c>
       <c r="B87" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C87" t="s">
         <v>131</v>
@@ -4539,7 +4539,7 @@
       </c>
       <c r="G87">
         <f t="shared" ca="1" si="9"/>
-        <v>999</v>
+        <v>1499</v>
       </c>
       <c r="H87">
         <f t="shared" si="10"/>
@@ -4564,7 +4564,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/khaki green formal trouser.avif</v>
       </c>
       <c r="B88" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C88" t="s">
         <v>143</v>
@@ -4580,14 +4580,14 @@
       </c>
       <c r="G88">
         <f t="shared" ca="1" si="9"/>
-        <v>1499</v>
+        <v>2899</v>
       </c>
       <c r="H88">
         <f t="shared" si="10"/>
         <v>1088</v>
       </c>
       <c r="I88" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J88">
         <v>6</v>
@@ -4605,7 +4605,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/light blue full sleeve shirt.avif</v>
       </c>
       <c r="B89" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C89" t="s">
         <v>142</v>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="G89">
         <f t="shared" ca="1" si="9"/>
-        <v>2299</v>
+        <v>1299</v>
       </c>
       <c r="H89">
         <f t="shared" si="10"/>
@@ -4646,7 +4646,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink flounced blouse.avif</v>
       </c>
       <c r="B90" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C90" t="s">
         <v>154</v>
@@ -4662,7 +4662,7 @@
       </c>
       <c r="G90">
         <f t="shared" ca="1" si="9"/>
-        <v>1899</v>
+        <v>4899</v>
       </c>
       <c r="H90">
         <f t="shared" si="10"/>
@@ -4687,7 +4687,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink tank top.avif</v>
       </c>
       <c r="B91" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C91" t="s">
         <v>154</v>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="G91">
         <f t="shared" ca="1" si="9"/>
-        <v>2999</v>
+        <v>1599</v>
       </c>
       <c r="H91">
         <f t="shared" si="10"/>
@@ -4728,7 +4728,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red fine knit.jpeg</v>
       </c>
       <c r="B92" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C92" t="s">
         <v>144</v>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="G92">
         <f t="shared" ca="1" si="9"/>
-        <v>1099</v>
+        <v>4699</v>
       </c>
       <c r="H92">
         <f t="shared" si="10"/>
@@ -4769,7 +4769,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red halter.avif</v>
       </c>
       <c r="B93" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C93" t="s">
         <v>144</v>
@@ -4785,7 +4785,7 @@
       </c>
       <c r="G93">
         <f t="shared" ca="1" si="9"/>
-        <v>2399</v>
+        <v>799</v>
       </c>
       <c r="H93">
         <f t="shared" si="10"/>
@@ -4810,7 +4810,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red peplum.avif</v>
       </c>
       <c r="B94" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C94" t="s">
         <v>144</v>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="G94">
         <f t="shared" ca="1" si="9"/>
-        <v>2199</v>
+        <v>4799</v>
       </c>
       <c r="H94">
         <f t="shared" si="10"/>
@@ -4851,7 +4851,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/white formal pants.avif</v>
       </c>
       <c r="B95" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C95" t="s">
         <v>115</v>
@@ -4860,21 +4860,21 @@
         <v>93</v>
       </c>
       <c r="E95" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F95" t="s">
         <v>115</v>
       </c>
       <c r="G95">
         <f t="shared" ca="1" si="9"/>
-        <v>1399</v>
+        <v>1699</v>
       </c>
       <c r="H95">
         <f t="shared" si="10"/>
         <v>1095</v>
       </c>
       <c r="I95" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J95">
         <v>6</v>
@@ -4892,7 +4892,7 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/yellow top.avif</v>
       </c>
       <c r="B96" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C96" t="s">
         <v>147</v>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="G96">
         <f t="shared" ca="1" si="9"/>
-        <v>3699</v>
+        <v>4199</v>
       </c>
       <c r="H96">
         <f t="shared" si="10"/>

</xml_diff>

<commit_message>
Added Supabase connection and DB test endpoint
</commit_message>
<xml_diff>
--- a/styleshop.xlsx
+++ b/styleshop.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aryanbhandari/aryancoding/styleshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881853F0-1212-9044-8797-7BA766872403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{751F7C32-55AE-BB49-879D-719BAD9BCAA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16100" xr2:uid="{296FE156-ABE8-A143-BE54-67E50949700F}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{296FE156-ABE8-A143-BE54-67E50949700F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$96</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="182">
   <si>
     <t>SKU</t>
   </si>
@@ -326,9 +326,6 @@
     <t>hangout</t>
   </si>
   <si>
-    <t xml:space="preserve">date, hangout </t>
-  </si>
-  <si>
     <t>hangout, date</t>
   </si>
   <si>
@@ -356,15 +353,6 @@
     <t>hangout,date,party</t>
   </si>
   <si>
-    <t>date,hangout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hangout,date </t>
-  </si>
-  <si>
-    <t>hangout,date</t>
-  </si>
-  <si>
     <t xml:space="preserve">date,party </t>
   </si>
   <si>
@@ -573,6 +561,30 @@
   </si>
   <si>
     <t>gender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date, casual  </t>
+  </si>
+  <si>
+    <t>casual , date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">casual </t>
+  </si>
+  <si>
+    <t>casual ,date,party</t>
+  </si>
+  <si>
+    <t xml:space="preserve">casual  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">date,casual </t>
+  </si>
+  <si>
+    <t xml:space="preserve">casual ,date </t>
+  </si>
+  <si>
+    <t>casual ,date</t>
   </si>
 </sst>
 </file>
@@ -963,13 +975,13 @@
         <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="F1" t="s">
         <v>7</v>
@@ -990,7 +1002,7 @@
         <v>6</v>
       </c>
       <c r="L1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -1002,20 +1014,20 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D2" t="s">
         <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G2">
         <f ca="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>1199</v>
+        <v>1599</v>
       </c>
       <c r="H2">
         <f>ROW()+1000</f>
@@ -1044,20 +1056,20 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D3" t="s">
         <v>92</v>
       </c>
       <c r="E3" t="s">
-        <v>95</v>
+        <v>174</v>
       </c>
       <c r="F3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G6" ca="1" si="1">RANDBETWEEN(7,19)*100+99</f>
-        <v>1399</v>
+        <v>799</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H66" si="2">ROW()+1000</f>
@@ -1086,20 +1098,20 @@
         <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D4" t="s">
         <v>92</v>
       </c>
       <c r="E4" t="s">
-        <v>95</v>
+        <v>174</v>
       </c>
       <c r="F4" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G4">
         <f t="shared" ca="1" si="1"/>
-        <v>1899</v>
+        <v>1099</v>
       </c>
       <c r="H4">
         <f t="shared" si="2"/>
@@ -1128,20 +1140,20 @@
         <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D5" t="s">
         <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G5">
         <f t="shared" ca="1" si="1"/>
-        <v>1199</v>
+        <v>1099</v>
       </c>
       <c r="H5">
         <f t="shared" si="2"/>
@@ -1170,16 +1182,16 @@
         <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D6" t="s">
         <v>92</v>
       </c>
       <c r="E6" t="s">
-        <v>96</v>
+        <v>175</v>
       </c>
       <c r="F6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G6">
         <f t="shared" ca="1" si="1"/>
@@ -1212,20 +1224,20 @@
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D7" t="s">
         <v>93</v>
       </c>
       <c r="E7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F7" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G7">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
-        <v>2599</v>
+        <v>4199</v>
       </c>
       <c r="H7">
         <f t="shared" si="2"/>
@@ -1254,20 +1266,20 @@
         <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
         <v>93</v>
       </c>
       <c r="E8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F8" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G8">
         <f t="shared" ref="G8:G13" ca="1" si="5">RANDBETWEEN(19,49)*100+99</f>
-        <v>4099</v>
+        <v>2999</v>
       </c>
       <c r="H8">
         <f t="shared" si="2"/>
@@ -1296,20 +1308,20 @@
         <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D9" t="s">
         <v>93</v>
       </c>
       <c r="E9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F9" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G9">
         <f t="shared" ca="1" si="5"/>
-        <v>2399</v>
+        <v>3099</v>
       </c>
       <c r="H9">
         <f t="shared" si="2"/>
@@ -1338,20 +1350,20 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D10" t="s">
         <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G10">
         <f t="shared" ca="1" si="5"/>
-        <v>4199</v>
+        <v>4299</v>
       </c>
       <c r="H10">
         <f t="shared" si="2"/>
@@ -1380,20 +1392,20 @@
         <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
         <v>93</v>
       </c>
       <c r="E11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F11" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G11">
         <f t="shared" ca="1" si="5"/>
-        <v>2499</v>
+        <v>3799</v>
       </c>
       <c r="H11">
         <f t="shared" si="2"/>
@@ -1422,20 +1434,20 @@
         <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D12" t="s">
         <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F12" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G12">
         <f ca="1">RANDBETWEEN(19,49)*100+99</f>
-        <v>4799</v>
+        <v>3599</v>
       </c>
       <c r="H12">
         <f t="shared" si="2"/>
@@ -1461,23 +1473,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/formalshirt_white.jpg</v>
       </c>
       <c r="B13" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
         <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F13" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G13">
         <f t="shared" ca="1" si="5"/>
-        <v>3399</v>
+        <v>4899</v>
       </c>
       <c r="H13">
         <f t="shared" si="2"/>
@@ -1506,27 +1518,27 @@
         <v>20</v>
       </c>
       <c r="C14" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
         <v>92</v>
       </c>
       <c r="E14" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F14" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G14">
         <f ca="1">RANDBETWEEN(7,49)*100+99</f>
-        <v>1799</v>
+        <v>2699</v>
       </c>
       <c r="H14">
         <f t="shared" si="2"/>
         <v>1014</v>
       </c>
       <c r="I14" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J14">
         <v>2</v>
@@ -1547,27 +1559,27 @@
         <v>21</v>
       </c>
       <c r="C15" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D15" t="s">
         <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F15" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G15">
         <f t="shared" ref="G15:G78" ca="1" si="6">RANDBETWEEN(7,49)*100+99</f>
-        <v>1999</v>
+        <v>3399</v>
       </c>
       <c r="H15">
         <f t="shared" si="2"/>
         <v>1015</v>
       </c>
       <c r="I15" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J15">
         <v>2</v>
@@ -1588,27 +1600,27 @@
         <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D16" t="s">
         <v>92</v>
       </c>
       <c r="E16" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F16" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G16">
         <f t="shared" ca="1" si="6"/>
-        <v>2999</v>
+        <v>799</v>
       </c>
       <c r="H16">
         <f t="shared" si="2"/>
         <v>1016</v>
       </c>
       <c r="I16" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J16">
         <v>2</v>
@@ -1629,27 +1641,27 @@
         <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D17" t="s">
         <v>92</v>
       </c>
       <c r="E17" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F17" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G17">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>799</v>
       </c>
       <c r="H17">
         <f t="shared" si="2"/>
         <v>1017</v>
       </c>
       <c r="I17" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J17">
         <v>2</v>
@@ -1670,27 +1682,27 @@
         <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D18" t="s">
         <v>92</v>
       </c>
       <c r="E18" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F18" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G18">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>2499</v>
       </c>
       <c r="H18">
         <f t="shared" si="2"/>
         <v>1018</v>
       </c>
       <c r="I18" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J18">
         <v>2</v>
@@ -1711,27 +1723,27 @@
         <v>25</v>
       </c>
       <c r="C19" t="s">
+        <v>111</v>
+      </c>
+      <c r="D19" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" t="s">
+        <v>176</v>
+      </c>
+      <c r="F19" t="s">
+        <v>111</v>
+      </c>
+      <c r="G19">
+        <f t="shared" ca="1" si="6"/>
+        <v>3399</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="2"/>
+        <v>1019</v>
+      </c>
+      <c r="I19" t="s">
         <v>115</v>
-      </c>
-      <c r="D19" t="s">
-        <v>92</v>
-      </c>
-      <c r="E19" t="s">
-        <v>94</v>
-      </c>
-      <c r="F19" t="s">
-        <v>115</v>
-      </c>
-      <c r="G19">
-        <f t="shared" ca="1" si="6"/>
-        <v>1799</v>
-      </c>
-      <c r="H19">
-        <f t="shared" si="2"/>
-        <v>1019</v>
-      </c>
-      <c r="I19" t="s">
-        <v>119</v>
       </c>
       <c r="J19">
         <v>4</v>
@@ -1752,20 +1764,20 @@
         <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D20" t="s">
         <v>92</v>
       </c>
       <c r="E20" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F20" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G20">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>899</v>
       </c>
       <c r="H20">
         <f t="shared" si="2"/>
@@ -1794,20 +1806,20 @@
         <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D21" t="s">
         <v>92</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F21" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G21">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>2099</v>
       </c>
       <c r="H21">
         <f t="shared" si="2"/>
@@ -1836,20 +1848,20 @@
         <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D22" t="s">
         <v>92</v>
       </c>
       <c r="E22" t="s">
-        <v>94</v>
+        <v>176</v>
       </c>
       <c r="F22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G22">
         <f t="shared" ca="1" si="6"/>
-        <v>4099</v>
+        <v>4699</v>
       </c>
       <c r="H22">
         <f t="shared" si="2"/>
@@ -1878,20 +1890,20 @@
         <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D23" t="s">
         <v>93</v>
       </c>
       <c r="E23" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G23">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>799</v>
       </c>
       <c r="H23">
         <f t="shared" si="2"/>
@@ -1920,20 +1932,20 @@
         <v>30</v>
       </c>
       <c r="C24" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D24" t="s">
         <v>93</v>
       </c>
       <c r="E24" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F24" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G24">
         <f t="shared" ca="1" si="6"/>
-        <v>2599</v>
+        <v>3799</v>
       </c>
       <c r="H24">
         <f t="shared" si="2"/>
@@ -1962,20 +1974,20 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="D25" t="s">
         <v>93</v>
       </c>
       <c r="E25" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F25" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G25">
         <f t="shared" ca="1" si="6"/>
-        <v>1999</v>
+        <v>3299</v>
       </c>
       <c r="H25">
         <f t="shared" si="2"/>
@@ -2004,20 +2016,20 @@
         <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D26" t="s">
         <v>93</v>
       </c>
       <c r="E26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F26" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G26">
         <f t="shared" ca="1" si="6"/>
-        <v>3599</v>
+        <v>1799</v>
       </c>
       <c r="H26">
         <f t="shared" si="2"/>
@@ -2046,20 +2058,20 @@
         <v>33</v>
       </c>
       <c r="C27" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D27" t="s">
         <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F27" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G27">
         <f t="shared" ca="1" si="6"/>
-        <v>4999</v>
+        <v>2399</v>
       </c>
       <c r="H27">
         <f t="shared" si="2"/>
@@ -2088,20 +2100,20 @@
         <v>34</v>
       </c>
       <c r="C28" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D28" t="s">
         <v>93</v>
       </c>
       <c r="E28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F28" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G28">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>899</v>
       </c>
       <c r="H28">
         <f t="shared" si="2"/>
@@ -2130,20 +2142,20 @@
         <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D29" t="s">
         <v>93</v>
       </c>
       <c r="E29" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F29" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G29">
         <f t="shared" ca="1" si="6"/>
-        <v>2399</v>
+        <v>4299</v>
       </c>
       <c r="H29">
         <f t="shared" si="2"/>
@@ -2172,20 +2184,20 @@
         <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D30" t="s">
         <v>92</v>
       </c>
       <c r="E30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F30" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G30">
         <f t="shared" ca="1" si="6"/>
-        <v>2199</v>
+        <v>3399</v>
       </c>
       <c r="H30">
         <f t="shared" si="2"/>
@@ -2214,20 +2226,20 @@
         <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D31" t="s">
         <v>92</v>
       </c>
       <c r="E31" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F31" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G31">
         <f t="shared" ca="1" si="6"/>
-        <v>4499</v>
+        <v>4099</v>
       </c>
       <c r="H31">
         <f t="shared" si="2"/>
@@ -2256,20 +2268,20 @@
         <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D32" t="s">
         <v>92</v>
       </c>
       <c r="E32" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F32" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G32">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>2399</v>
       </c>
       <c r="H32">
         <f t="shared" si="2"/>
@@ -2298,20 +2310,20 @@
         <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D33" t="s">
         <v>92</v>
       </c>
       <c r="E33" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F33" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G33">
         <f t="shared" ca="1" si="6"/>
-        <v>2899</v>
+        <v>2999</v>
       </c>
       <c r="H33">
         <f t="shared" si="2"/>
@@ -2340,20 +2352,20 @@
         <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D34" t="s">
         <v>92</v>
       </c>
       <c r="E34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F34" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G34">
         <f t="shared" ca="1" si="6"/>
-        <v>2599</v>
+        <v>4599</v>
       </c>
       <c r="H34">
         <f t="shared" si="2"/>
@@ -2382,20 +2394,20 @@
         <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D35" t="s">
         <v>92</v>
       </c>
       <c r="E35" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F35" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G35">
         <f t="shared" ca="1" si="6"/>
-        <v>899</v>
+        <v>2599</v>
       </c>
       <c r="H35">
         <f t="shared" si="2"/>
@@ -2424,16 +2436,16 @@
         <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D36" t="s">
         <v>92</v>
       </c>
       <c r="E36" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F36" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G36">
         <f t="shared" ca="1" si="6"/>
@@ -2466,7 +2478,7 @@
         <v>43</v>
       </c>
       <c r="C37" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D37" t="s">
         <v>93</v>
@@ -2475,11 +2487,11 @@
         <v>94</v>
       </c>
       <c r="F37" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G37">
         <f t="shared" ca="1" si="6"/>
-        <v>2699</v>
+        <v>2199</v>
       </c>
       <c r="H37">
         <f t="shared" si="2"/>
@@ -2508,20 +2520,20 @@
         <v>44</v>
       </c>
       <c r="C38" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D38" t="s">
         <v>93</v>
       </c>
       <c r="E38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F38" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G38">
         <f t="shared" ca="1" si="6"/>
-        <v>2299</v>
+        <v>4099</v>
       </c>
       <c r="H38">
         <f t="shared" si="2"/>
@@ -2550,20 +2562,20 @@
         <v>45</v>
       </c>
       <c r="C39" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D39" t="s">
         <v>93</v>
       </c>
       <c r="E39" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F39" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G39">
         <f t="shared" ca="1" si="6"/>
-        <v>4999</v>
+        <v>3099</v>
       </c>
       <c r="H39">
         <f t="shared" si="2"/>
@@ -2592,27 +2604,27 @@
         <v>46</v>
       </c>
       <c r="C40" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D40" t="s">
         <v>92</v>
       </c>
       <c r="E40" t="s">
-        <v>104</v>
+        <v>177</v>
       </c>
       <c r="F40" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G40">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>2799</v>
       </c>
       <c r="H40">
         <f t="shared" si="2"/>
         <v>1040</v>
       </c>
       <c r="I40" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J40">
         <v>7</v>
@@ -2633,27 +2645,27 @@
         <v>47</v>
       </c>
       <c r="C41" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D41" t="s">
         <v>92</v>
       </c>
       <c r="E41" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F41" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G41">
         <f t="shared" ca="1" si="6"/>
-        <v>3799</v>
+        <v>3299</v>
       </c>
       <c r="H41">
         <f t="shared" si="2"/>
         <v>1041</v>
       </c>
       <c r="I41" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J41">
         <v>7</v>
@@ -2674,27 +2686,27 @@
         <v>48</v>
       </c>
       <c r="C42" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D42" t="s">
         <v>92</v>
       </c>
       <c r="E42" t="s">
-        <v>104</v>
+        <v>177</v>
       </c>
       <c r="F42" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G42">
         <f t="shared" ca="1" si="6"/>
-        <v>4999</v>
+        <v>3999</v>
       </c>
       <c r="H42">
         <f t="shared" si="2"/>
         <v>1042</v>
       </c>
       <c r="I42" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J42">
         <v>7</v>
@@ -2715,27 +2727,27 @@
         <v>49</v>
       </c>
       <c r="C43" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D43" t="s">
         <v>92</v>
       </c>
       <c r="E43" t="s">
-        <v>105</v>
+        <v>179</v>
       </c>
       <c r="F43" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G43">
         <f t="shared" ca="1" si="6"/>
-        <v>2599</v>
+        <v>1499</v>
       </c>
       <c r="H43">
         <f t="shared" si="2"/>
         <v>1043</v>
       </c>
       <c r="I43" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J43">
         <v>7</v>
@@ -2756,27 +2768,27 @@
         <v>50</v>
       </c>
       <c r="C44" t="s">
+        <v>111</v>
+      </c>
+      <c r="D44" t="s">
+        <v>92</v>
+      </c>
+      <c r="E44" t="s">
+        <v>179</v>
+      </c>
+      <c r="F44" t="s">
+        <v>111</v>
+      </c>
+      <c r="G44">
+        <f t="shared" ca="1" si="6"/>
+        <v>2999</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="2"/>
+        <v>1044</v>
+      </c>
+      <c r="I44" t="s">
         <v>115</v>
-      </c>
-      <c r="D44" t="s">
-        <v>92</v>
-      </c>
-      <c r="E44" t="s">
-        <v>105</v>
-      </c>
-      <c r="F44" t="s">
-        <v>115</v>
-      </c>
-      <c r="G44">
-        <f t="shared" ca="1" si="6"/>
-        <v>2099</v>
-      </c>
-      <c r="H44">
-        <f t="shared" si="2"/>
-        <v>1044</v>
-      </c>
-      <c r="I44" t="s">
-        <v>119</v>
       </c>
       <c r="J44">
         <v>5</v>
@@ -2797,20 +2809,20 @@
         <v>51</v>
       </c>
       <c r="C45" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D45" t="s">
         <v>92</v>
       </c>
       <c r="E45" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F45" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G45">
         <f t="shared" ca="1" si="6"/>
-        <v>4999</v>
+        <v>1299</v>
       </c>
       <c r="H45">
         <f t="shared" si="2"/>
@@ -2839,20 +2851,20 @@
         <v>52</v>
       </c>
       <c r="C46" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D46" t="s">
         <v>92</v>
       </c>
       <c r="E46" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F46" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G46">
         <f t="shared" ca="1" si="6"/>
-        <v>999</v>
+        <v>1899</v>
       </c>
       <c r="H46">
         <f t="shared" si="2"/>
@@ -2881,20 +2893,20 @@
         <v>53</v>
       </c>
       <c r="C47" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D47" t="s">
         <v>92</v>
       </c>
       <c r="E47" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F47" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G47">
         <f t="shared" ca="1" si="6"/>
-        <v>4999</v>
+        <v>1999</v>
       </c>
       <c r="H47">
         <f t="shared" si="2"/>
@@ -2923,27 +2935,27 @@
         <v>54</v>
       </c>
       <c r="C48" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D48" t="s">
         <v>92</v>
       </c>
       <c r="E48" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F48" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G48">
         <f t="shared" ca="1" si="6"/>
-        <v>2999</v>
+        <v>1499</v>
       </c>
       <c r="H48">
         <f t="shared" si="2"/>
         <v>1048</v>
       </c>
       <c r="I48" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="J48">
         <v>5</v>
@@ -2964,27 +2976,27 @@
         <v>55</v>
       </c>
       <c r="C49" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D49" t="s">
         <v>92</v>
       </c>
       <c r="E49" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F49" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G49">
         <f t="shared" ca="1" si="6"/>
-        <v>999</v>
+        <v>3399</v>
       </c>
       <c r="H49">
         <f t="shared" si="2"/>
         <v>1049</v>
       </c>
       <c r="I49" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="J49">
         <v>5</v>
@@ -3005,20 +3017,20 @@
         <v>56</v>
       </c>
       <c r="C50" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D50" t="s">
         <v>92</v>
       </c>
       <c r="E50" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F50" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G50">
         <f t="shared" ca="1" si="6"/>
-        <v>2499</v>
+        <v>4199</v>
       </c>
       <c r="H50">
         <f t="shared" si="2"/>
@@ -3047,20 +3059,20 @@
         <v>57</v>
       </c>
       <c r="C51" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D51" t="s">
         <v>92</v>
       </c>
       <c r="E51" t="s">
-        <v>106</v>
+        <v>180</v>
       </c>
       <c r="F51" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G51">
         <f t="shared" ca="1" si="6"/>
-        <v>2199</v>
+        <v>4699</v>
       </c>
       <c r="H51">
         <f t="shared" si="2"/>
@@ -3089,20 +3101,20 @@
         <v>58</v>
       </c>
       <c r="C52" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D52" t="s">
         <v>92</v>
       </c>
       <c r="E52" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F52" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G52">
         <f t="shared" ca="1" si="6"/>
-        <v>4499</v>
+        <v>3299</v>
       </c>
       <c r="H52">
         <f t="shared" si="2"/>
@@ -3131,20 +3143,20 @@
         <v>59</v>
       </c>
       <c r="C53" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D53" t="s">
         <v>92</v>
       </c>
       <c r="E53" t="s">
-        <v>107</v>
+        <v>181</v>
       </c>
       <c r="F53" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G53">
         <f t="shared" ca="1" si="6"/>
-        <v>1499</v>
+        <v>4699</v>
       </c>
       <c r="H53">
         <f t="shared" si="2"/>
@@ -3173,20 +3185,20 @@
         <v>60</v>
       </c>
       <c r="C54" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D54" t="s">
         <v>92</v>
       </c>
       <c r="E54" t="s">
-        <v>95</v>
+        <v>174</v>
       </c>
       <c r="F54" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G54">
         <f t="shared" ca="1" si="6"/>
-        <v>2599</v>
+        <v>3999</v>
       </c>
       <c r="H54">
         <f t="shared" si="2"/>
@@ -3214,27 +3226,27 @@
         <v>61</v>
       </c>
       <c r="C55" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D55" t="s">
         <v>92</v>
       </c>
       <c r="E55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F55" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G55">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>4699</v>
       </c>
       <c r="H55">
         <f t="shared" si="2"/>
         <v>1055</v>
       </c>
       <c r="I55" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J55">
         <v>5</v>
@@ -3255,27 +3267,27 @@
         <v>62</v>
       </c>
       <c r="C56" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D56" t="s">
         <v>92</v>
       </c>
       <c r="E56" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F56" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G56">
         <f t="shared" ca="1" si="6"/>
-        <v>3199</v>
+        <v>3399</v>
       </c>
       <c r="H56">
         <f t="shared" si="2"/>
         <v>1056</v>
       </c>
       <c r="I56" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J56">
         <v>5</v>
@@ -3296,27 +3308,27 @@
         <v>63</v>
       </c>
       <c r="C57" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D57" t="s">
         <v>92</v>
       </c>
       <c r="E57" t="s">
+        <v>104</v>
+      </c>
+      <c r="F57" t="s">
         <v>108</v>
       </c>
-      <c r="F57" t="s">
-        <v>112</v>
-      </c>
       <c r="G57">
         <f t="shared" ca="1" si="6"/>
-        <v>3899</v>
+        <v>4299</v>
       </c>
       <c r="H57">
         <f t="shared" si="2"/>
         <v>1057</v>
       </c>
       <c r="I57" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J57">
         <v>5</v>
@@ -3337,27 +3349,27 @@
         <v>64</v>
       </c>
       <c r="C58" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D58" t="s">
         <v>92</v>
       </c>
       <c r="E58" t="s">
-        <v>96</v>
+        <v>175</v>
       </c>
       <c r="F58" t="s">
+        <v>113</v>
+      </c>
+      <c r="G58">
+        <f t="shared" ca="1" si="6"/>
+        <v>4099</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="2"/>
+        <v>1058</v>
+      </c>
+      <c r="I58" t="s">
         <v>117</v>
-      </c>
-      <c r="G58">
-        <f t="shared" ca="1" si="6"/>
-        <v>3899</v>
-      </c>
-      <c r="H58">
-        <f t="shared" si="2"/>
-        <v>1058</v>
-      </c>
-      <c r="I58" t="s">
-        <v>121</v>
       </c>
       <c r="J58">
         <v>5</v>
@@ -3378,27 +3390,27 @@
         <v>65</v>
       </c>
       <c r="C59" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D59" t="s">
         <v>92</v>
       </c>
       <c r="E59" t="s">
-        <v>105</v>
+        <v>179</v>
       </c>
       <c r="F59" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G59">
         <f t="shared" ca="1" si="6"/>
-        <v>4599</v>
+        <v>799</v>
       </c>
       <c r="H59">
         <f t="shared" si="2"/>
         <v>1059</v>
       </c>
       <c r="I59" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J59">
         <v>5</v>
@@ -3419,27 +3431,27 @@
         <v>66</v>
       </c>
       <c r="C60" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D60" t="s">
         <v>93</v>
       </c>
       <c r="E60" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F60" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G60">
         <f t="shared" ca="1" si="6"/>
-        <v>999</v>
+        <v>4199</v>
       </c>
       <c r="H60">
         <f t="shared" si="2"/>
         <v>1060</v>
       </c>
       <c r="I60" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="J60">
         <v>3</v>
@@ -3460,27 +3472,27 @@
         <v>67</v>
       </c>
       <c r="C61" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D61" t="s">
         <v>92</v>
       </c>
       <c r="E61" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F61" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G61">
         <f t="shared" ca="1" si="6"/>
-        <v>2699</v>
+        <v>1499</v>
       </c>
       <c r="H61">
         <f t="shared" si="2"/>
         <v>1061</v>
       </c>
       <c r="I61" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J61">
         <v>3</v>
@@ -3501,27 +3513,27 @@
         <v>68</v>
       </c>
       <c r="C62" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D62" t="s">
         <v>92</v>
       </c>
       <c r="E62" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F62" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G62">
         <f t="shared" ca="1" si="6"/>
-        <v>3499</v>
+        <v>1999</v>
       </c>
       <c r="H62">
         <f t="shared" si="2"/>
         <v>1062</v>
       </c>
       <c r="I62" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="J62">
         <v>3</v>
@@ -3542,27 +3554,27 @@
         <v>69</v>
       </c>
       <c r="C63" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D63" t="s">
         <v>92</v>
       </c>
       <c r="E63" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F63" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G63">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>1799</v>
       </c>
       <c r="H63">
         <f t="shared" si="2"/>
         <v>1063</v>
       </c>
       <c r="I63" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J63">
         <v>3</v>
@@ -3583,20 +3595,20 @@
         <v>70</v>
       </c>
       <c r="C64" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D64" t="s">
         <v>93</v>
       </c>
       <c r="E64" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F64" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G64">
         <f t="shared" ca="1" si="6"/>
-        <v>3699</v>
+        <v>4899</v>
       </c>
       <c r="H64">
         <f t="shared" si="2"/>
@@ -3624,20 +3636,20 @@
         <v>71</v>
       </c>
       <c r="C65" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D65" t="s">
         <v>93</v>
       </c>
       <c r="E65" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F65" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G65">
         <f t="shared" ca="1" si="6"/>
-        <v>2099</v>
+        <v>3099</v>
       </c>
       <c r="H65">
         <f t="shared" si="2"/>
@@ -3665,20 +3677,20 @@
         <v>72</v>
       </c>
       <c r="C66" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D66" t="s">
         <v>92</v>
       </c>
       <c r="E66" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F66" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G66">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>2099</v>
       </c>
       <c r="H66">
         <f t="shared" si="2"/>
@@ -3706,20 +3718,20 @@
         <v>73</v>
       </c>
       <c r="C67" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D67" t="s">
         <v>93</v>
       </c>
       <c r="E67" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F67" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G67">
         <f t="shared" ca="1" si="6"/>
-        <v>4799</v>
+        <v>3099</v>
       </c>
       <c r="H67">
         <f t="shared" ref="H67:H79" si="7">ROW()+1000</f>
@@ -3747,20 +3759,20 @@
         <v>74</v>
       </c>
       <c r="C68" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D68" t="s">
         <v>92</v>
       </c>
       <c r="E68" t="s">
-        <v>104</v>
+        <v>177</v>
       </c>
       <c r="F68" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G68">
         <f t="shared" ca="1" si="6"/>
-        <v>4699</v>
+        <v>999</v>
       </c>
       <c r="H68">
         <f t="shared" si="7"/>
@@ -3788,7 +3800,7 @@
         <v>75</v>
       </c>
       <c r="C69" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D69" t="s">
         <v>93</v>
@@ -3797,11 +3809,11 @@
         <v>94</v>
       </c>
       <c r="F69" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G69">
         <f t="shared" ca="1" si="6"/>
-        <v>1799</v>
+        <v>2699</v>
       </c>
       <c r="H69">
         <f t="shared" si="7"/>
@@ -3829,20 +3841,20 @@
         <v>76</v>
       </c>
       <c r="C70" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D70" t="s">
         <v>93</v>
       </c>
       <c r="E70" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F70" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G70">
         <f t="shared" ca="1" si="6"/>
-        <v>1399</v>
+        <v>2599</v>
       </c>
       <c r="H70">
         <f t="shared" si="7"/>
@@ -3870,27 +3882,27 @@
         <v>77</v>
       </c>
       <c r="C71" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D71" t="s">
         <v>92</v>
       </c>
       <c r="E71" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F71" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G71">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>3899</v>
       </c>
       <c r="H71">
         <f t="shared" si="7"/>
         <v>1071</v>
       </c>
       <c r="I71" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="J71">
         <v>3</v>
@@ -3911,27 +3923,27 @@
         <v>78</v>
       </c>
       <c r="C72" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D72" t="s">
         <v>92</v>
       </c>
       <c r="E72" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F72" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G72">
         <f t="shared" ca="1" si="6"/>
-        <v>799</v>
+        <v>4899</v>
       </c>
       <c r="H72">
         <f t="shared" si="7"/>
         <v>1072</v>
       </c>
       <c r="I72" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="J72">
         <v>3</v>
@@ -3952,27 +3964,27 @@
         <v>79</v>
       </c>
       <c r="C73" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D73" t="s">
         <v>93</v>
       </c>
       <c r="E73" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F73" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G73">
         <f t="shared" ca="1" si="6"/>
-        <v>4099</v>
+        <v>4799</v>
       </c>
       <c r="H73">
         <f t="shared" si="7"/>
         <v>1073</v>
       </c>
       <c r="I73" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="J73">
         <v>3</v>
@@ -3993,27 +4005,27 @@
         <v>80</v>
       </c>
       <c r="C74" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D74" t="s">
         <v>92</v>
       </c>
       <c r="E74" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F74" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G74">
         <f t="shared" ca="1" si="6"/>
-        <v>1599</v>
+        <v>4499</v>
       </c>
       <c r="H74">
         <f t="shared" si="7"/>
         <v>1074</v>
       </c>
       <c r="I74" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J74">
         <v>3</v>
@@ -4034,20 +4046,20 @@
         <v>81</v>
       </c>
       <c r="C75" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D75" t="s">
         <v>92</v>
       </c>
       <c r="E75" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F75" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G75">
         <f t="shared" ca="1" si="6"/>
-        <v>4699</v>
+        <v>4199</v>
       </c>
       <c r="H75">
         <f t="shared" si="7"/>
@@ -4075,20 +4087,20 @@
         <v>82</v>
       </c>
       <c r="C76" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D76" t="s">
         <v>92</v>
       </c>
       <c r="E76" t="s">
-        <v>104</v>
+        <v>177</v>
       </c>
       <c r="F76" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G76">
         <f t="shared" ca="1" si="6"/>
-        <v>3099</v>
+        <v>2499</v>
       </c>
       <c r="H76">
         <f t="shared" si="7"/>
@@ -4116,20 +4128,20 @@
         <v>83</v>
       </c>
       <c r="C77" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D77" t="s">
         <v>93</v>
       </c>
       <c r="E77" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F77" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G77">
         <f t="shared" ca="1" si="6"/>
-        <v>4099</v>
+        <v>2099</v>
       </c>
       <c r="H77">
         <f t="shared" si="7"/>
@@ -4157,20 +4169,20 @@
         <v>84</v>
       </c>
       <c r="C78" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D78" t="s">
         <v>92</v>
       </c>
       <c r="E78" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F78" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G78">
         <f t="shared" ca="1" si="6"/>
-        <v>4399</v>
+        <v>3699</v>
       </c>
       <c r="H78">
         <f t="shared" si="7"/>
@@ -4198,27 +4210,27 @@
         <v>85</v>
       </c>
       <c r="C79" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D79" t="s">
         <v>92</v>
       </c>
       <c r="E79" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F79" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G79">
         <f t="shared" ref="G79:G96" ca="1" si="9">RANDBETWEEN(7,49)*100+99</f>
-        <v>1299</v>
+        <v>799</v>
       </c>
       <c r="H79">
         <f t="shared" si="7"/>
         <v>1079</v>
       </c>
       <c r="I79" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J79">
         <v>6</v>
@@ -4239,7 +4251,7 @@
         <v>86</v>
       </c>
       <c r="C80" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D80" t="s">
         <v>93</v>
@@ -4248,18 +4260,18 @@
         <v>94</v>
       </c>
       <c r="F80" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G80">
         <f t="shared" ca="1" si="9"/>
-        <v>2799</v>
+        <v>3499</v>
       </c>
       <c r="H80">
         <f>ROW()+1000</f>
         <v>1080</v>
       </c>
       <c r="I80" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="J80">
         <v>6</v>
@@ -4280,27 +4292,27 @@
         <v>87</v>
       </c>
       <c r="C81" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D81" t="s">
         <v>92</v>
       </c>
       <c r="E81" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F81" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G81">
         <f t="shared" ca="1" si="9"/>
-        <v>3199</v>
+        <v>1299</v>
       </c>
       <c r="H81">
         <f t="shared" ref="H81:H96" si="10">ROW()+1000</f>
         <v>1081</v>
       </c>
       <c r="I81" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J81">
         <v>6</v>
@@ -4321,27 +4333,27 @@
         <v>88</v>
       </c>
       <c r="C82" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D82" t="s">
         <v>92</v>
       </c>
       <c r="E82" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F82" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G82">
         <f t="shared" ca="1" si="9"/>
-        <v>3199</v>
+        <v>899</v>
       </c>
       <c r="H82">
         <f t="shared" si="10"/>
         <v>1082</v>
       </c>
       <c r="I82" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J82">
         <v>6</v>
@@ -4362,27 +4374,27 @@
         <v>89</v>
       </c>
       <c r="C83" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D83" t="s">
         <v>92</v>
       </c>
       <c r="E83" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F83" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G83">
         <f t="shared" ca="1" si="9"/>
-        <v>1599</v>
+        <v>4499</v>
       </c>
       <c r="H83">
         <f t="shared" si="10"/>
         <v>1083</v>
       </c>
       <c r="I83" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="J83">
         <v>6</v>
@@ -4394,36 +4406,36 @@
         <v>91</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="str">
         <f t="shared" si="8"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/black formal pants.avif</v>
       </c>
       <c r="B84" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C84" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D84" t="s">
         <v>93</v>
       </c>
       <c r="E84" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="F84" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G84">
         <f t="shared" ca="1" si="9"/>
-        <v>4699</v>
+        <v>3899</v>
       </c>
       <c r="H84">
         <f t="shared" si="10"/>
         <v>1084</v>
       </c>
       <c r="I84" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J84">
         <v>6</v>
@@ -4441,23 +4453,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue croptop.avif</v>
       </c>
       <c r="B85" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C85" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D85" t="s">
         <v>92</v>
       </c>
       <c r="E85" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F85" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G85">
         <f t="shared" ca="1" si="9"/>
-        <v>4399</v>
+        <v>1499</v>
       </c>
       <c r="H85">
         <f t="shared" si="10"/>
@@ -4476,7 +4488,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" t="str">
         <f t="shared" si="8"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/blue jeans.avif</v>
@@ -4485,20 +4497,20 @@
         <v>66</v>
       </c>
       <c r="C86" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D86" t="s">
         <v>93</v>
       </c>
       <c r="E86" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F86" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="G86">
         <f t="shared" ca="1" si="9"/>
-        <v>2099</v>
+        <v>2599</v>
       </c>
       <c r="H86">
         <f t="shared" si="10"/>
@@ -4523,23 +4535,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/halter neck sequined.avif</v>
       </c>
       <c r="B87" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C87" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D87" t="s">
         <v>92</v>
       </c>
       <c r="E87" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F87" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G87">
         <f t="shared" ca="1" si="9"/>
-        <v>1799</v>
+        <v>4999</v>
       </c>
       <c r="H87">
         <f t="shared" si="10"/>
@@ -4558,36 +4570,36 @@
         <v>91</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="str">
         <f t="shared" si="8"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/khaki green formal trouser.avif</v>
       </c>
       <c r="B88" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C88" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D88" t="s">
         <v>93</v>
       </c>
       <c r="E88" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F88" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G88">
         <f t="shared" ca="1" si="9"/>
-        <v>2999</v>
+        <v>899</v>
       </c>
       <c r="H88">
         <f t="shared" si="10"/>
         <v>1088</v>
       </c>
       <c r="I88" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J88">
         <v>6</v>
@@ -4605,23 +4617,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/light blue full sleeve shirt.avif</v>
       </c>
       <c r="B89" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C89" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D89" t="s">
         <v>92</v>
       </c>
       <c r="E89" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F89" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G89">
         <f t="shared" ca="1" si="9"/>
-        <v>2799</v>
+        <v>4699</v>
       </c>
       <c r="H89">
         <f t="shared" si="10"/>
@@ -4646,23 +4658,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink flounced blouse.avif</v>
       </c>
       <c r="B90" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C90" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D90" t="s">
         <v>92</v>
       </c>
       <c r="E90" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F90" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G90">
         <f t="shared" ca="1" si="9"/>
-        <v>999</v>
+        <v>2899</v>
       </c>
       <c r="H90">
         <f t="shared" si="10"/>
@@ -4687,23 +4699,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/pink tank top.avif</v>
       </c>
       <c r="B91" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="C91" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D91" t="s">
         <v>92</v>
       </c>
       <c r="E91" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F91" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="G91">
         <f t="shared" ca="1" si="9"/>
-        <v>1399</v>
+        <v>2199</v>
       </c>
       <c r="H91">
         <f t="shared" si="10"/>
@@ -4728,23 +4740,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red fine knit.jpeg</v>
       </c>
       <c r="B92" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C92" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D92" t="s">
         <v>92</v>
       </c>
       <c r="E92" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F92" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G92">
         <f t="shared" ca="1" si="9"/>
-        <v>1799</v>
+        <v>3199</v>
       </c>
       <c r="H92">
         <f t="shared" si="10"/>
@@ -4769,23 +4781,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red halter.avif</v>
       </c>
       <c r="B93" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C93" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D93" t="s">
         <v>92</v>
       </c>
       <c r="E93" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F93" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G93">
         <f t="shared" ca="1" si="9"/>
-        <v>2399</v>
+        <v>3299</v>
       </c>
       <c r="H93">
         <f t="shared" si="10"/>
@@ -4810,19 +4822,19 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/red peplum.avif</v>
       </c>
       <c r="B94" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C94" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="D94" t="s">
         <v>92</v>
       </c>
       <c r="E94" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F94" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G94">
         <f t="shared" ca="1" si="9"/>
@@ -4845,36 +4857,36 @@
         <v>91</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" t="str">
         <f t="shared" si="8"/>
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/white formal pants.avif</v>
       </c>
       <c r="B95" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C95" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D95" t="s">
         <v>93</v>
       </c>
       <c r="E95" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="F95" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G95">
         <f t="shared" ca="1" si="9"/>
-        <v>2599</v>
+        <v>4599</v>
       </c>
       <c r="H95">
         <f t="shared" si="10"/>
         <v>1095</v>
       </c>
       <c r="I95" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J95">
         <v>6</v>
@@ -4892,23 +4904,23 @@
         <v>https://onodppswtexnqmgyegdo.supabase.co/storage/v1/object/public/demo_images/yellow top.avif</v>
       </c>
       <c r="B96" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C96" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D96" t="s">
         <v>92</v>
       </c>
       <c r="E96" t="s">
-        <v>103</v>
+        <v>178</v>
       </c>
       <c r="F96" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G96">
         <f t="shared" ca="1" si="9"/>
-        <v>4599</v>
+        <v>1999</v>
       </c>
       <c r="H96">
         <f t="shared" si="10"/>
@@ -4928,7 +4940,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{BC477210-8802-4647-A9A0-82022E3B188B}">
+  <autoFilter ref="A1:K96" xr:uid="{BC477210-8802-4647-A9A0-82022E3B188B}">
     <filterColumn colId="3">
       <filters>
         <filter val="top"/>

</xml_diff>